<commit_message>
Update mapping workbook for latest ClearOps fields file
ProjectManualCreation was removed upstream; adjust summary accordingly.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A5mSLBPV7GuwkbXJCnEXu9
</commit_message>
<xml_diff>
--- a/ClearOps_Database_Mapped.xlsx
+++ b/ClearOps_Database_Mapped.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issues_Fixed" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Table_Catalog'!$A$1:$E$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Columns_Corrected'!$A$1:$G$388</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Table_Catalog'!$A$1:$E$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Columns_Corrected'!$A$1:$G$387</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'FK_Mapping'!$A$1:$F$55</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Issues_Fixed'!$A$1:$D$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Issues_Fixed'!$A$1:$D$81</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -493,14 +493,14 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Source: 28 tables across 4 groups (Setup 7, TimePlanner 3, Project 7, Admin 11).</t>
+          <t>Source (latest upload): 27 tables across 4 groups (Setup 7, TimePlanner 3, Project 6, Admin 11). Compared with the previous upload, the only change is that ProjectManualCreation was removed; every other table is identical.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Result: 33 tables in the corrected model = 25 kept/fixed + 5 new + 3 retired (merged).</t>
+          <t>Result: 32 tables in the corrected model = 25 kept/fixed + 5 new + 2 to retire (still in your file; ProjectManualCreation is already gone).</t>
         </is>
       </c>
     </row>
@@ -538,7 +538,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>3. Duplicate tables: ProjectManualCreation duplicated Project_Master; RolesandPermissions duplicated Role/Page/Permission/Users; ProjectForecasting duplicated ProjectSTP. All retired/merged.</t>
+          <t>3. Duplicate tables: ProjectManualCreation (now removed from your file, good) duplicated Project_Master, so manual creation is covered by Project_Master.Source; RolesandPermissions duplicated Role/Page/Permission/Users; ProjectForecasting duplicated ProjectSTP. ProjectForecasting and RolesandPermissions are still in your file and should be retired.</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1249,30 +1249,34 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>ProjectManualCreation</t>
+          <t>Admin_IntegrationStatus</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Project</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>Merged</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr"/>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Sys_Integration_Id</t>
+        </is>
+      </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>RETIRED: field-for-field duplicate of Project_Master. Use Project_Master.Source='MANUAL'</t>
+          <t>Integration status per source system</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Admin_IntegrationStatus</t>
+          <t>ClearOps_Logs</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1287,19 +1291,19 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Sys_Integration_Id</t>
+          <t>Log_Id</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Integration status per source system</t>
+          <t>Integration/cron run log (was Logs_table)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_Logs</t>
+          <t>ClearOps_Role</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
@@ -1314,19 +1318,19 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Log_Id</t>
+          <t>Role_Id</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Integration/cron run log (was Logs_table)</t>
+          <t>Role master</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_Role</t>
+          <t>ClearOps_Page</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -1341,19 +1345,19 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Role_Id</t>
+          <t>Page_Id</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Role master</t>
+          <t>Application pages/screens</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_Page</t>
+          <t>ClearOps_Access</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -1368,19 +1372,19 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Page_Id</t>
+          <t>Access_Id</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Application pages/screens</t>
+          <t>Access level lookup: None / R / R/W</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_Access</t>
+          <t>ClearOps_Permission</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
@@ -1395,19 +1399,19 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Access_Id</t>
+          <t>Permission_Id</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Access level lookup: None / R / R/W</t>
+          <t>Role x Page -&gt; access level (mapping table)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_Permission</t>
+          <t>ClearOps_Users</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -1422,19 +1426,19 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Permission_Id</t>
+          <t>User_Id</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Role x Page -&gt; access level (mapping table)</t>
+          <t>Application users</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_Users</t>
+          <t>ClearOps_Login</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -1449,19 +1453,19 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>User_Id</t>
+          <t>Login_Id</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Application users</t>
+          <t>SSO identity mapping</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_Login</t>
+          <t>ClearOps_UserLogin</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
@@ -1476,19 +1480,19 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Login_Id</t>
+          <t>User_Login_Id</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>SSO identity mapping</t>
+          <t>Login event history</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_UserLogin</t>
+          <t>RolesandPermissions</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -1496,47 +1500,20 @@
           <t>Admin</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>Fixed</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>User_Login_Id</t>
-        </is>
-      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Merged</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr"/>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Login event history</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>RolesandPermissions</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Admin</t>
-        </is>
-      </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>Merged</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
           <t>RETIRED: denormalised sheet of Role+Page+Permission+Users. Replace with a VIEW</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E34"/>
+  <autoFilter ref="A1:E33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1547,7 +1524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G388"/>
+  <dimension ref="A1:G387"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -10358,27 +10335,31 @@
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>ProjectManualCreation</t>
+          <t>Admin_IntegrationStatus</t>
         </is>
       </c>
       <c r="B313" s="2" t="inlineStr">
         <is>
-          <t>All columns</t>
-        </is>
-      </c>
-      <c r="C313" s="2" t="inlineStr"/>
-      <c r="D313" s="2" t="inlineStr"/>
+          <t>Sys_Integration_Id</t>
+        </is>
+      </c>
+      <c r="C313" s="2" t="inlineStr">
+        <is>
+          <t>BIGINT</t>
+        </is>
+      </c>
+      <c r="D313" s="2" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
       <c r="E313" s="2" t="inlineStr"/>
-      <c r="F313" s="7" t="inlineStr">
-        <is>
-          <t>Moved/Removed</t>
-        </is>
-      </c>
-      <c r="G313" s="2" t="inlineStr">
-        <is>
-          <t>Duplicate of Project_Master</t>
-        </is>
-      </c>
+      <c r="F313" s="2" t="inlineStr">
+        <is>
+          <t>Kept</t>
+        </is>
+      </c>
+      <c r="G313" s="2" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
@@ -10388,26 +10369,26 @@
       </c>
       <c r="B314" s="2" t="inlineStr">
         <is>
-          <t>Sys_Integration_Id</t>
+          <t>System_Name</t>
         </is>
       </c>
       <c r="C314" s="2" t="inlineStr">
         <is>
-          <t>BIGINT</t>
-        </is>
-      </c>
-      <c r="D314" s="2" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
+          <t>VARCHAR(100)</t>
+        </is>
+      </c>
+      <c r="D314" s="2" t="inlineStr"/>
       <c r="E314" s="2" t="inlineStr"/>
-      <c r="F314" s="2" t="inlineStr">
-        <is>
-          <t>Kept</t>
-        </is>
-      </c>
-      <c r="G314" s="2" t="inlineStr"/>
+      <c r="F314" s="5" t="inlineStr">
+        <is>
+          <t>Renamed</t>
+        </is>
+      </c>
+      <c r="G314" s="2" t="inlineStr">
+        <is>
+          <t>Was System</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" s="2" t="inlineStr">
@@ -10417,26 +10398,22 @@
       </c>
       <c r="B315" s="2" t="inlineStr">
         <is>
-          <t>System_Name</t>
+          <t>Last_Sync_DateTime</t>
         </is>
       </c>
       <c r="C315" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
+          <t>DATETIME2</t>
         </is>
       </c>
       <c r="D315" s="2" t="inlineStr"/>
       <c r="E315" s="2" t="inlineStr"/>
-      <c r="F315" s="5" t="inlineStr">
-        <is>
-          <t>Renamed</t>
-        </is>
-      </c>
-      <c r="G315" s="2" t="inlineStr">
-        <is>
-          <t>Was System</t>
-        </is>
-      </c>
+      <c r="F315" s="2" t="inlineStr">
+        <is>
+          <t>Kept</t>
+        </is>
+      </c>
+      <c r="G315" s="2" t="inlineStr"/>
     </row>
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
@@ -10446,12 +10423,12 @@
       </c>
       <c r="B316" s="2" t="inlineStr">
         <is>
-          <t>Last_Sync_DateTime</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="C316" s="2" t="inlineStr">
         <is>
-          <t>DATETIME2</t>
+          <t>VARCHAR(20)</t>
         </is>
       </c>
       <c r="D316" s="2" t="inlineStr"/>
@@ -10471,22 +10448,26 @@
       </c>
       <c r="B317" s="2" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Records_Captured</t>
         </is>
       </c>
       <c r="C317" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(20)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D317" s="2" t="inlineStr"/>
       <c r="E317" s="2" t="inlineStr"/>
-      <c r="F317" s="2" t="inlineStr">
-        <is>
-          <t>Kept</t>
-        </is>
-      </c>
-      <c r="G317" s="2" t="inlineStr"/>
+      <c r="F317" s="5" t="inlineStr">
+        <is>
+          <t>Renamed</t>
+        </is>
+      </c>
+      <c r="G317" s="2" t="inlineStr">
+        <is>
+          <t>Was record_captured</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" s="2" t="inlineStr">
@@ -10496,24 +10477,24 @@
       </c>
       <c r="B318" s="2" t="inlineStr">
         <is>
-          <t>Records_Captured</t>
+          <t>Created_By</t>
         </is>
       </c>
       <c r="C318" s="2" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="D318" s="2" t="inlineStr"/>
       <c r="E318" s="2" t="inlineStr"/>
-      <c r="F318" s="5" t="inlineStr">
-        <is>
-          <t>Renamed</t>
+      <c r="F318" s="2" t="inlineStr">
+        <is>
+          <t>Kept</t>
         </is>
       </c>
       <c r="G318" s="2" t="inlineStr">
         <is>
-          <t>Was record_captured</t>
+          <t>Audit column</t>
         </is>
       </c>
     </row>
@@ -10525,12 +10506,12 @@
       </c>
       <c r="B319" s="2" t="inlineStr">
         <is>
-          <t>Created_By</t>
+          <t>Created_Date</t>
         </is>
       </c>
       <c r="C319" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
+          <t>DATETIME2</t>
         </is>
       </c>
       <c r="D319" s="2" t="inlineStr"/>
@@ -10554,12 +10535,12 @@
       </c>
       <c r="B320" s="2" t="inlineStr">
         <is>
-          <t>Created_Date</t>
+          <t>Modified_By</t>
         </is>
       </c>
       <c r="C320" s="2" t="inlineStr">
         <is>
-          <t>DATETIME2</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="D320" s="2" t="inlineStr"/>
@@ -10583,12 +10564,12 @@
       </c>
       <c r="B321" s="2" t="inlineStr">
         <is>
-          <t>Modified_By</t>
+          <t>Modified_Date</t>
         </is>
       </c>
       <c r="C321" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
+          <t>DATETIME2</t>
         </is>
       </c>
       <c r="D321" s="2" t="inlineStr"/>
@@ -10607,31 +10588,31 @@
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>Admin_IntegrationStatus</t>
+          <t>ClearOps_Logs</t>
         </is>
       </c>
       <c r="B322" s="2" t="inlineStr">
         <is>
-          <t>Modified_Date</t>
+          <t>Log_Id</t>
         </is>
       </c>
       <c r="C322" s="2" t="inlineStr">
         <is>
-          <t>DATETIME2</t>
-        </is>
-      </c>
-      <c r="D322" s="2" t="inlineStr"/>
+          <t>BIGINT</t>
+        </is>
+      </c>
+      <c r="D322" s="2" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
       <c r="E322" s="2" t="inlineStr"/>
       <c r="F322" s="2" t="inlineStr">
         <is>
           <t>Kept</t>
         </is>
       </c>
-      <c r="G322" s="2" t="inlineStr">
-        <is>
-          <t>Audit column</t>
-        </is>
-      </c>
+      <c r="G322" s="2" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
@@ -10641,7 +10622,7 @@
       </c>
       <c r="B323" s="2" t="inlineStr">
         <is>
-          <t>Log_Id</t>
+          <t>Sys_Integration_Id</t>
         </is>
       </c>
       <c r="C323" s="2" t="inlineStr">
@@ -10651,10 +10632,14 @@
       </c>
       <c r="D323" s="2" t="inlineStr">
         <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="E323" s="2" t="inlineStr"/>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="E323" s="2" t="inlineStr">
+        <is>
+          <t>Admin_IntegrationStatus.Sys_Integration_Id</t>
+        </is>
+      </c>
       <c r="F323" s="2" t="inlineStr">
         <is>
           <t>Kept</t>
@@ -10670,30 +10655,26 @@
       </c>
       <c r="B324" s="2" t="inlineStr">
         <is>
-          <t>Sys_Integration_Id</t>
+          <t>Cron_Job_Run_Id</t>
         </is>
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>BIGINT</t>
-        </is>
-      </c>
-      <c r="D324" s="2" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="E324" s="2" t="inlineStr">
-        <is>
-          <t>Admin_IntegrationStatus.Sys_Integration_Id</t>
-        </is>
-      </c>
-      <c r="F324" s="2" t="inlineStr">
-        <is>
-          <t>Kept</t>
-        </is>
-      </c>
-      <c r="G324" s="2" t="inlineStr"/>
+          <t>VARCHAR(50)</t>
+        </is>
+      </c>
+      <c r="D324" s="2" t="inlineStr"/>
+      <c r="E324" s="2" t="inlineStr"/>
+      <c r="F324" s="5" t="inlineStr">
+        <is>
+          <t>Renamed</t>
+        </is>
+      </c>
+      <c r="G324" s="2" t="inlineStr">
+        <is>
+          <t>Was cornjob run_id (typo)</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
@@ -10703,24 +10684,24 @@
       </c>
       <c r="B325" s="2" t="inlineStr">
         <is>
-          <t>Cron_Job_Run_Id</t>
+          <t>Run_Start</t>
         </is>
       </c>
       <c r="C325" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(50)</t>
+          <t>DATETIME2</t>
         </is>
       </c>
       <c r="D325" s="2" t="inlineStr"/>
       <c r="E325" s="2" t="inlineStr"/>
-      <c r="F325" s="5" t="inlineStr">
-        <is>
-          <t>Renamed</t>
+      <c r="F325" s="6" t="inlineStr">
+        <is>
+          <t>Added</t>
         </is>
       </c>
       <c r="G325" s="2" t="inlineStr">
         <is>
-          <t>Was cornjob run_id (typo)</t>
+          <t>MISSING</t>
         </is>
       </c>
     </row>
@@ -10732,7 +10713,7 @@
       </c>
       <c r="B326" s="2" t="inlineStr">
         <is>
-          <t>Run_Start</t>
+          <t>Run_End</t>
         </is>
       </c>
       <c r="C326" s="2" t="inlineStr">
@@ -10761,12 +10742,12 @@
       </c>
       <c r="B327" s="2" t="inlineStr">
         <is>
-          <t>Run_End</t>
+          <t>Run_Status</t>
         </is>
       </c>
       <c r="C327" s="2" t="inlineStr">
         <is>
-          <t>DATETIME2</t>
+          <t>VARCHAR(20)</t>
         </is>
       </c>
       <c r="D327" s="2" t="inlineStr"/>
@@ -10790,12 +10771,12 @@
       </c>
       <c r="B328" s="2" t="inlineStr">
         <is>
-          <t>Run_Status</t>
+          <t>Records_Processed</t>
         </is>
       </c>
       <c r="C328" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(20)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D328" s="2" t="inlineStr"/>
@@ -10819,12 +10800,12 @@
       </c>
       <c r="B329" s="2" t="inlineStr">
         <is>
-          <t>Records_Processed</t>
+          <t>Error_Message</t>
         </is>
       </c>
       <c r="C329" s="2" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>VARCHAR(2000)</t>
         </is>
       </c>
       <c r="D329" s="2" t="inlineStr"/>
@@ -10848,12 +10829,12 @@
       </c>
       <c r="B330" s="2" t="inlineStr">
         <is>
-          <t>Error_Message</t>
+          <t>Created_By</t>
         </is>
       </c>
       <c r="C330" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(2000)</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="D330" s="2" t="inlineStr"/>
@@ -10865,7 +10846,7 @@
       </c>
       <c r="G330" s="2" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>Audit column (MISSING in sheet)</t>
         </is>
       </c>
     </row>
@@ -10877,12 +10858,12 @@
       </c>
       <c r="B331" s="2" t="inlineStr">
         <is>
-          <t>Created_By</t>
+          <t>Created_Date</t>
         </is>
       </c>
       <c r="C331" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
+          <t>DATETIME2</t>
         </is>
       </c>
       <c r="D331" s="2" t="inlineStr"/>
@@ -10906,12 +10887,12 @@
       </c>
       <c r="B332" s="2" t="inlineStr">
         <is>
-          <t>Created_Date</t>
+          <t>Modified_By</t>
         </is>
       </c>
       <c r="C332" s="2" t="inlineStr">
         <is>
-          <t>DATETIME2</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="D332" s="2" t="inlineStr"/>
@@ -10935,12 +10916,12 @@
       </c>
       <c r="B333" s="2" t="inlineStr">
         <is>
-          <t>Modified_By</t>
+          <t>Modified_Date</t>
         </is>
       </c>
       <c r="C333" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
+          <t>DATETIME2</t>
         </is>
       </c>
       <c r="D333" s="2" t="inlineStr"/>
@@ -10959,31 +10940,31 @@
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_Logs</t>
+          <t>ClearOps_Role</t>
         </is>
       </c>
       <c r="B334" s="2" t="inlineStr">
         <is>
-          <t>Modified_Date</t>
+          <t>Role_Id</t>
         </is>
       </c>
       <c r="C334" s="2" t="inlineStr">
         <is>
-          <t>DATETIME2</t>
-        </is>
-      </c>
-      <c r="D334" s="2" t="inlineStr"/>
+          <t>BIGINT</t>
+        </is>
+      </c>
+      <c r="D334" s="2" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
       <c r="E334" s="2" t="inlineStr"/>
-      <c r="F334" s="6" t="inlineStr">
-        <is>
-          <t>Added</t>
-        </is>
-      </c>
-      <c r="G334" s="2" t="inlineStr">
-        <is>
-          <t>Audit column (MISSING in sheet)</t>
-        </is>
-      </c>
+      <c r="F334" s="2" t="inlineStr">
+        <is>
+          <t>Kept</t>
+        </is>
+      </c>
+      <c r="G334" s="2" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
@@ -10993,19 +10974,15 @@
       </c>
       <c r="B335" s="2" t="inlineStr">
         <is>
-          <t>Role_Id</t>
+          <t>Role_Name</t>
         </is>
       </c>
       <c r="C335" s="2" t="inlineStr">
         <is>
-          <t>BIGINT</t>
-        </is>
-      </c>
-      <c r="D335" s="2" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
+          <t>VARCHAR(100)</t>
+        </is>
+      </c>
+      <c r="D335" s="2" t="inlineStr"/>
       <c r="E335" s="2" t="inlineStr"/>
       <c r="F335" s="2" t="inlineStr">
         <is>
@@ -11022,12 +10999,12 @@
       </c>
       <c r="B336" s="2" t="inlineStr">
         <is>
-          <t>Role_Name</t>
+          <t>Role_Type</t>
         </is>
       </c>
       <c r="C336" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
+          <t>VARCHAR(30)</t>
         </is>
       </c>
       <c r="D336" s="2" t="inlineStr"/>
@@ -11047,22 +11024,26 @@
       </c>
       <c r="B337" s="2" t="inlineStr">
         <is>
-          <t>Role_Type</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="C337" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(30)</t>
+          <t>VARCHAR(20)</t>
         </is>
       </c>
       <c r="D337" s="2" t="inlineStr"/>
       <c r="E337" s="2" t="inlineStr"/>
-      <c r="F337" s="2" t="inlineStr">
-        <is>
-          <t>Kept</t>
-        </is>
-      </c>
-      <c r="G337" s="2" t="inlineStr"/>
+      <c r="F337" s="6" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="G337" s="2" t="inlineStr">
+        <is>
+          <t>From RolesandPermissions</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
@@ -11072,24 +11053,24 @@
       </c>
       <c r="B338" s="2" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Created_By</t>
         </is>
       </c>
       <c r="C338" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(20)</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="D338" s="2" t="inlineStr"/>
       <c r="E338" s="2" t="inlineStr"/>
-      <c r="F338" s="6" t="inlineStr">
-        <is>
-          <t>Added</t>
+      <c r="F338" s="2" t="inlineStr">
+        <is>
+          <t>Kept</t>
         </is>
       </c>
       <c r="G338" s="2" t="inlineStr">
         <is>
-          <t>From RolesandPermissions</t>
+          <t>Audit column</t>
         </is>
       </c>
     </row>
@@ -11101,12 +11082,12 @@
       </c>
       <c r="B339" s="2" t="inlineStr">
         <is>
-          <t>Created_By</t>
+          <t>Created_Date</t>
         </is>
       </c>
       <c r="C339" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
+          <t>DATETIME2</t>
         </is>
       </c>
       <c r="D339" s="2" t="inlineStr"/>
@@ -11130,12 +11111,12 @@
       </c>
       <c r="B340" s="2" t="inlineStr">
         <is>
-          <t>Created_Date</t>
+          <t>Modified_By</t>
         </is>
       </c>
       <c r="C340" s="2" t="inlineStr">
         <is>
-          <t>DATETIME2</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="D340" s="2" t="inlineStr"/>
@@ -11159,12 +11140,12 @@
       </c>
       <c r="B341" s="2" t="inlineStr">
         <is>
-          <t>Modified_By</t>
+          <t>Modified_Date</t>
         </is>
       </c>
       <c r="C341" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
+          <t>DATETIME2</t>
         </is>
       </c>
       <c r="D341" s="2" t="inlineStr"/>
@@ -11183,31 +11164,31 @@
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_Role</t>
+          <t>ClearOps_Page</t>
         </is>
       </c>
       <c r="B342" s="2" t="inlineStr">
         <is>
-          <t>Modified_Date</t>
+          <t>Page_Id</t>
         </is>
       </c>
       <c r="C342" s="2" t="inlineStr">
         <is>
-          <t>DATETIME2</t>
-        </is>
-      </c>
-      <c r="D342" s="2" t="inlineStr"/>
+          <t>BIGINT</t>
+        </is>
+      </c>
+      <c r="D342" s="2" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
       <c r="E342" s="2" t="inlineStr"/>
       <c r="F342" s="2" t="inlineStr">
         <is>
           <t>Kept</t>
         </is>
       </c>
-      <c r="G342" s="2" t="inlineStr">
-        <is>
-          <t>Audit column</t>
-        </is>
-      </c>
+      <c r="G342" s="2" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" s="2" t="inlineStr">
@@ -11217,19 +11198,15 @@
       </c>
       <c r="B343" s="2" t="inlineStr">
         <is>
-          <t>Page_Id</t>
+          <t>Page_Number</t>
         </is>
       </c>
       <c r="C343" s="2" t="inlineStr">
         <is>
-          <t>BIGINT</t>
-        </is>
-      </c>
-      <c r="D343" s="2" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
+          <t>INT</t>
+        </is>
+      </c>
+      <c r="D343" s="2" t="inlineStr"/>
       <c r="E343" s="2" t="inlineStr"/>
       <c r="F343" s="2" t="inlineStr">
         <is>
@@ -11246,12 +11223,12 @@
       </c>
       <c r="B344" s="2" t="inlineStr">
         <is>
-          <t>Page_Number</t>
+          <t>Page_Name</t>
         </is>
       </c>
       <c r="C344" s="2" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>VARCHAR(150)</t>
         </is>
       </c>
       <c r="D344" s="2" t="inlineStr"/>
@@ -11271,22 +11248,26 @@
       </c>
       <c r="B345" s="2" t="inlineStr">
         <is>
-          <t>Page_Name</t>
+          <t>Module</t>
         </is>
       </c>
       <c r="C345" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(150)</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="D345" s="2" t="inlineStr"/>
       <c r="E345" s="2" t="inlineStr"/>
-      <c r="F345" s="2" t="inlineStr">
-        <is>
-          <t>Kept</t>
-        </is>
-      </c>
-      <c r="G345" s="2" t="inlineStr"/>
+      <c r="F345" s="6" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="G345" s="2" t="inlineStr">
+        <is>
+          <t>Moved from RolesandPermissions</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
@@ -11296,7 +11277,7 @@
       </c>
       <c r="B346" s="2" t="inlineStr">
         <is>
-          <t>Module</t>
+          <t>Created_By</t>
         </is>
       </c>
       <c r="C346" s="2" t="inlineStr">
@@ -11306,14 +11287,14 @@
       </c>
       <c r="D346" s="2" t="inlineStr"/>
       <c r="E346" s="2" t="inlineStr"/>
-      <c r="F346" s="6" t="inlineStr">
-        <is>
-          <t>Added</t>
+      <c r="F346" s="2" t="inlineStr">
+        <is>
+          <t>Kept</t>
         </is>
       </c>
       <c r="G346" s="2" t="inlineStr">
         <is>
-          <t>Moved from RolesandPermissions</t>
+          <t>Audit column</t>
         </is>
       </c>
     </row>
@@ -11325,12 +11306,12 @@
       </c>
       <c r="B347" s="2" t="inlineStr">
         <is>
-          <t>Created_By</t>
+          <t>Created_Date</t>
         </is>
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
+          <t>DATETIME2</t>
         </is>
       </c>
       <c r="D347" s="2" t="inlineStr"/>
@@ -11354,12 +11335,12 @@
       </c>
       <c r="B348" s="2" t="inlineStr">
         <is>
-          <t>Created_Date</t>
+          <t>Modified_By</t>
         </is>
       </c>
       <c r="C348" s="2" t="inlineStr">
         <is>
-          <t>DATETIME2</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="D348" s="2" t="inlineStr"/>
@@ -11383,12 +11364,12 @@
       </c>
       <c r="B349" s="2" t="inlineStr">
         <is>
-          <t>Modified_By</t>
+          <t>Modified_Date</t>
         </is>
       </c>
       <c r="C349" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
+          <t>DATETIME2</t>
         </is>
       </c>
       <c r="D349" s="2" t="inlineStr"/>
@@ -11407,31 +11388,31 @@
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_Page</t>
+          <t>ClearOps_Access</t>
         </is>
       </c>
       <c r="B350" s="2" t="inlineStr">
         <is>
-          <t>Modified_Date</t>
+          <t>Access_Id</t>
         </is>
       </c>
       <c r="C350" s="2" t="inlineStr">
         <is>
-          <t>DATETIME2</t>
-        </is>
-      </c>
-      <c r="D350" s="2" t="inlineStr"/>
+          <t>BIGINT</t>
+        </is>
+      </c>
+      <c r="D350" s="2" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
       <c r="E350" s="2" t="inlineStr"/>
       <c r="F350" s="2" t="inlineStr">
         <is>
           <t>Kept</t>
         </is>
       </c>
-      <c r="G350" s="2" t="inlineStr">
-        <is>
-          <t>Audit column</t>
-        </is>
-      </c>
+      <c r="G350" s="2" t="inlineStr"/>
     </row>
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
@@ -11441,26 +11422,26 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>Access_Id</t>
+          <t>Access_Type</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>BIGINT</t>
-        </is>
-      </c>
-      <c r="D351" s="2" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
+          <t>VARCHAR(10)</t>
+        </is>
+      </c>
+      <c r="D351" s="2" t="inlineStr"/>
       <c r="E351" s="2" t="inlineStr"/>
-      <c r="F351" s="2" t="inlineStr">
-        <is>
-          <t>Kept</t>
-        </is>
-      </c>
-      <c r="G351" s="2" t="inlineStr"/>
+      <c r="F351" s="5" t="inlineStr">
+        <is>
+          <t>Renamed</t>
+        </is>
+      </c>
+      <c r="G351" s="2" t="inlineStr">
+        <is>
+          <t>Was Accrss_type (typo)</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
@@ -11470,24 +11451,24 @@
       </c>
       <c r="B352" s="2" t="inlineStr">
         <is>
-          <t>Access_Type</t>
+          <t>Created_By</t>
         </is>
       </c>
       <c r="C352" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(10)</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="D352" s="2" t="inlineStr"/>
       <c r="E352" s="2" t="inlineStr"/>
-      <c r="F352" s="5" t="inlineStr">
-        <is>
-          <t>Renamed</t>
+      <c r="F352" s="2" t="inlineStr">
+        <is>
+          <t>Kept</t>
         </is>
       </c>
       <c r="G352" s="2" t="inlineStr">
         <is>
-          <t>Was Accrss_type (typo)</t>
+          <t>Audit column</t>
         </is>
       </c>
     </row>
@@ -11499,12 +11480,12 @@
       </c>
       <c r="B353" s="2" t="inlineStr">
         <is>
-          <t>Created_By</t>
+          <t>Created_Date</t>
         </is>
       </c>
       <c r="C353" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
+          <t>DATETIME2</t>
         </is>
       </c>
       <c r="D353" s="2" t="inlineStr"/>
@@ -11528,12 +11509,12 @@
       </c>
       <c r="B354" s="2" t="inlineStr">
         <is>
-          <t>Created_Date</t>
+          <t>Modified_By</t>
         </is>
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>DATETIME2</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="D354" s="2" t="inlineStr"/>
@@ -11557,12 +11538,12 @@
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>Modified_By</t>
+          <t>Modified_Date</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
+          <t>DATETIME2</t>
         </is>
       </c>
       <c r="D355" s="2" t="inlineStr"/>
@@ -11581,31 +11562,31 @@
     <row r="356">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_Access</t>
+          <t>ClearOps_Permission</t>
         </is>
       </c>
       <c r="B356" s="2" t="inlineStr">
         <is>
-          <t>Modified_Date</t>
+          <t>Permission_Id</t>
         </is>
       </c>
       <c r="C356" s="2" t="inlineStr">
         <is>
-          <t>DATETIME2</t>
-        </is>
-      </c>
-      <c r="D356" s="2" t="inlineStr"/>
+          <t>BIGINT</t>
+        </is>
+      </c>
+      <c r="D356" s="2" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
       <c r="E356" s="2" t="inlineStr"/>
       <c r="F356" s="2" t="inlineStr">
         <is>
           <t>Kept</t>
         </is>
       </c>
-      <c r="G356" s="2" t="inlineStr">
-        <is>
-          <t>Audit column</t>
-        </is>
-      </c>
+      <c r="G356" s="2" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" s="2" t="inlineStr">
@@ -11615,7 +11596,7 @@
       </c>
       <c r="B357" s="2" t="inlineStr">
         <is>
-          <t>Permission_Id</t>
+          <t>Role_Id</t>
         </is>
       </c>
       <c r="C357" s="2" t="inlineStr">
@@ -11625,10 +11606,14 @@
       </c>
       <c r="D357" s="2" t="inlineStr">
         <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="E357" s="2" t="inlineStr"/>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="E357" s="2" t="inlineStr">
+        <is>
+          <t>ClearOps_Role.Role_Id</t>
+        </is>
+      </c>
       <c r="F357" s="2" t="inlineStr">
         <is>
           <t>Kept</t>
@@ -11644,7 +11629,7 @@
       </c>
       <c r="B358" s="2" t="inlineStr">
         <is>
-          <t>Role_Id</t>
+          <t>Page_Id</t>
         </is>
       </c>
       <c r="C358" s="2" t="inlineStr">
@@ -11659,7 +11644,7 @@
       </c>
       <c r="E358" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_Role.Role_Id</t>
+          <t>ClearOps_Page.Page_Id</t>
         </is>
       </c>
       <c r="F358" s="2" t="inlineStr">
@@ -11677,7 +11662,7 @@
       </c>
       <c r="B359" s="2" t="inlineStr">
         <is>
-          <t>Page_Id</t>
+          <t>Access_Id</t>
         </is>
       </c>
       <c r="C359" s="2" t="inlineStr">
@@ -11692,7 +11677,7 @@
       </c>
       <c r="E359" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_Page.Page_Id</t>
+          <t>ClearOps_Access.Access_Id</t>
         </is>
       </c>
       <c r="F359" s="2" t="inlineStr">
@@ -11710,30 +11695,22 @@
       </c>
       <c r="B360" s="2" t="inlineStr">
         <is>
-          <t>Access_Id</t>
-        </is>
-      </c>
-      <c r="C360" s="2" t="inlineStr">
-        <is>
-          <t>BIGINT</t>
-        </is>
-      </c>
-      <c r="D360" s="2" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="E360" s="2" t="inlineStr">
-        <is>
-          <t>ClearOps_Access.Access_Id</t>
-        </is>
-      </c>
-      <c r="F360" s="2" t="inlineStr">
-        <is>
-          <t>Kept</t>
-        </is>
-      </c>
-      <c r="G360" s="2" t="inlineStr"/>
+          <t>HRID</t>
+        </is>
+      </c>
+      <c r="C360" s="2" t="inlineStr"/>
+      <c r="D360" s="2" t="inlineStr"/>
+      <c r="E360" s="2" t="inlineStr"/>
+      <c r="F360" s="7" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="G360" s="2" t="inlineStr">
+        <is>
+          <t>A role permission is not per person; user-&gt;role is in ClearOps_Users</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
@@ -11743,20 +11720,24 @@
       </c>
       <c r="B361" s="2" t="inlineStr">
         <is>
-          <t>HRID</t>
-        </is>
-      </c>
-      <c r="C361" s="2" t="inlineStr"/>
+          <t>Created_By</t>
+        </is>
+      </c>
+      <c r="C361" s="2" t="inlineStr">
+        <is>
+          <t>VARCHAR(100)</t>
+        </is>
+      </c>
       <c r="D361" s="2" t="inlineStr"/>
       <c r="E361" s="2" t="inlineStr"/>
-      <c r="F361" s="7" t="inlineStr">
-        <is>
-          <t>Removed</t>
+      <c r="F361" s="2" t="inlineStr">
+        <is>
+          <t>Kept</t>
         </is>
       </c>
       <c r="G361" s="2" t="inlineStr">
         <is>
-          <t>A role permission is not per person; user-&gt;role is in ClearOps_Users</t>
+          <t>Audit column</t>
         </is>
       </c>
     </row>
@@ -11768,12 +11749,12 @@
       </c>
       <c r="B362" s="2" t="inlineStr">
         <is>
-          <t>Created_By</t>
+          <t>Created_Date</t>
         </is>
       </c>
       <c r="C362" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
+          <t>DATETIME2</t>
         </is>
       </c>
       <c r="D362" s="2" t="inlineStr"/>
@@ -11797,12 +11778,12 @@
       </c>
       <c r="B363" s="2" t="inlineStr">
         <is>
-          <t>Created_Date</t>
+          <t>Modified_By</t>
         </is>
       </c>
       <c r="C363" s="2" t="inlineStr">
         <is>
-          <t>DATETIME2</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="D363" s="2" t="inlineStr"/>
@@ -11826,12 +11807,12 @@
       </c>
       <c r="B364" s="2" t="inlineStr">
         <is>
-          <t>Modified_By</t>
+          <t>Modified_Date</t>
         </is>
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
+          <t>DATETIME2</t>
         </is>
       </c>
       <c r="D364" s="2" t="inlineStr"/>
@@ -11850,29 +11831,33 @@
     <row r="365">
       <c r="A365" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_Permission</t>
+          <t>ClearOps_Users</t>
         </is>
       </c>
       <c r="B365" s="2" t="inlineStr">
         <is>
-          <t>Modified_Date</t>
+          <t>User_Id</t>
         </is>
       </c>
       <c r="C365" s="2" t="inlineStr">
         <is>
-          <t>DATETIME2</t>
-        </is>
-      </c>
-      <c r="D365" s="2" t="inlineStr"/>
+          <t>BIGINT</t>
+        </is>
+      </c>
+      <c r="D365" s="2" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
       <c r="E365" s="2" t="inlineStr"/>
-      <c r="F365" s="2" t="inlineStr">
-        <is>
-          <t>Kept</t>
+      <c r="F365" s="5" t="inlineStr">
+        <is>
+          <t>Renamed</t>
         </is>
       </c>
       <c r="G365" s="2" t="inlineStr">
         <is>
-          <t>Audit column</t>
+          <t>Was User_ID(PK) (sr_id)</t>
         </is>
       </c>
     </row>
@@ -11884,28 +11869,32 @@
       </c>
       <c r="B366" s="2" t="inlineStr">
         <is>
-          <t>User_Id</t>
+          <t>HRID</t>
         </is>
       </c>
       <c r="C366" s="2" t="inlineStr">
         <is>
-          <t>BIGINT</t>
+          <t>VARCHAR(20)</t>
         </is>
       </c>
       <c r="D366" s="2" t="inlineStr">
         <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="E366" s="2" t="inlineStr"/>
-      <c r="F366" s="5" t="inlineStr">
-        <is>
-          <t>Renamed</t>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="E366" s="2" t="inlineStr">
+        <is>
+          <t>Employee_Master.HRID</t>
+        </is>
+      </c>
+      <c r="F366" s="2" t="inlineStr">
+        <is>
+          <t>Kept</t>
         </is>
       </c>
       <c r="G366" s="2" t="inlineStr">
         <is>
-          <t>Was User_ID(PK) (sr_id)</t>
+          <t>UNIQUE</t>
         </is>
       </c>
     </row>
@@ -11917,12 +11906,12 @@
       </c>
       <c r="B367" s="2" t="inlineStr">
         <is>
-          <t>HRID</t>
+          <t>Role_Id</t>
         </is>
       </c>
       <c r="C367" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(20)</t>
+          <t>BIGINT</t>
         </is>
       </c>
       <c r="D367" s="2" t="inlineStr">
@@ -11932,7 +11921,7 @@
       </c>
       <c r="E367" s="2" t="inlineStr">
         <is>
-          <t>Employee_Master.HRID</t>
+          <t>ClearOps_Role.Role_Id</t>
         </is>
       </c>
       <c r="F367" s="2" t="inlineStr">
@@ -11940,11 +11929,7 @@
           <t>Kept</t>
         </is>
       </c>
-      <c r="G367" s="2" t="inlineStr">
-        <is>
-          <t>UNIQUE</t>
-        </is>
-      </c>
+      <c r="G367" s="2" t="inlineStr"/>
     </row>
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
@@ -11954,27 +11939,19 @@
       </c>
       <c r="B368" s="2" t="inlineStr">
         <is>
-          <t>Role_Id</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="C368" s="2" t="inlineStr">
         <is>
-          <t>BIGINT</t>
-        </is>
-      </c>
-      <c r="D368" s="2" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="E368" s="2" t="inlineStr">
-        <is>
-          <t>ClearOps_Role.Role_Id</t>
-        </is>
-      </c>
-      <c r="F368" s="2" t="inlineStr">
-        <is>
-          <t>Kept</t>
+          <t>VARCHAR(20)</t>
+        </is>
+      </c>
+      <c r="D368" s="2" t="inlineStr"/>
+      <c r="E368" s="2" t="inlineStr"/>
+      <c r="F368" s="6" t="inlineStr">
+        <is>
+          <t>Added</t>
         </is>
       </c>
       <c r="G368" s="2" t="inlineStr"/>
@@ -11987,22 +11964,22 @@
       </c>
       <c r="B369" s="2" t="inlineStr">
         <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C369" s="2" t="inlineStr">
-        <is>
-          <t>VARCHAR(20)</t>
-        </is>
-      </c>
+          <t>Role_Name, Name, Email</t>
+        </is>
+      </c>
+      <c r="C369" s="2" t="inlineStr"/>
       <c r="D369" s="2" t="inlineStr"/>
       <c r="E369" s="2" t="inlineStr"/>
-      <c r="F369" s="6" t="inlineStr">
-        <is>
-          <t>Added</t>
-        </is>
-      </c>
-      <c r="G369" s="2" t="inlineStr"/>
+      <c r="F369" s="7" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="G369" s="2" t="inlineStr">
+        <is>
+          <t>Derivable via Role_Id / HRID</t>
+        </is>
+      </c>
     </row>
     <row r="370">
       <c r="A370" s="2" t="inlineStr">
@@ -12012,20 +11989,24 @@
       </c>
       <c r="B370" s="2" t="inlineStr">
         <is>
-          <t>Role_Name, Name, Email</t>
-        </is>
-      </c>
-      <c r="C370" s="2" t="inlineStr"/>
+          <t>Created_By</t>
+        </is>
+      </c>
+      <c r="C370" s="2" t="inlineStr">
+        <is>
+          <t>VARCHAR(100)</t>
+        </is>
+      </c>
       <c r="D370" s="2" t="inlineStr"/>
       <c r="E370" s="2" t="inlineStr"/>
-      <c r="F370" s="7" t="inlineStr">
-        <is>
-          <t>Removed</t>
+      <c r="F370" s="2" t="inlineStr">
+        <is>
+          <t>Kept</t>
         </is>
       </c>
       <c r="G370" s="2" t="inlineStr">
         <is>
-          <t>Derivable via Role_Id / HRID</t>
+          <t>Audit column</t>
         </is>
       </c>
     </row>
@@ -12037,12 +12018,12 @@
       </c>
       <c r="B371" s="2" t="inlineStr">
         <is>
-          <t>Created_By</t>
+          <t>Created_Date</t>
         </is>
       </c>
       <c r="C371" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
+          <t>DATETIME2</t>
         </is>
       </c>
       <c r="D371" s="2" t="inlineStr"/>
@@ -12066,12 +12047,12 @@
       </c>
       <c r="B372" s="2" t="inlineStr">
         <is>
-          <t>Created_Date</t>
+          <t>Modified_By</t>
         </is>
       </c>
       <c r="C372" s="2" t="inlineStr">
         <is>
-          <t>DATETIME2</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="D372" s="2" t="inlineStr"/>
@@ -12095,12 +12076,12 @@
       </c>
       <c r="B373" s="2" t="inlineStr">
         <is>
-          <t>Modified_By</t>
+          <t>Modified_Date</t>
         </is>
       </c>
       <c r="C373" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
+          <t>DATETIME2</t>
         </is>
       </c>
       <c r="D373" s="2" t="inlineStr"/>
@@ -12119,29 +12100,33 @@
     <row r="374">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_Users</t>
+          <t>ClearOps_Login</t>
         </is>
       </c>
       <c r="B374" s="2" t="inlineStr">
         <is>
-          <t>Modified_Date</t>
+          <t>Login_Id</t>
         </is>
       </c>
       <c r="C374" s="2" t="inlineStr">
         <is>
-          <t>DATETIME2</t>
-        </is>
-      </c>
-      <c r="D374" s="2" t="inlineStr"/>
+          <t>BIGINT</t>
+        </is>
+      </c>
+      <c r="D374" s="2" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
       <c r="E374" s="2" t="inlineStr"/>
-      <c r="F374" s="2" t="inlineStr">
-        <is>
-          <t>Kept</t>
+      <c r="F374" s="6" t="inlineStr">
+        <is>
+          <t>Added</t>
         </is>
       </c>
       <c r="G374" s="2" t="inlineStr">
         <is>
-          <t>Audit column</t>
+          <t>MISSING: table had no PK</t>
         </is>
       </c>
     </row>
@@ -12153,30 +12138,30 @@
       </c>
       <c r="B375" s="2" t="inlineStr">
         <is>
-          <t>Login_Id</t>
+          <t>HRID</t>
         </is>
       </c>
       <c r="C375" s="2" t="inlineStr">
         <is>
-          <t>BIGINT</t>
+          <t>VARCHAR(20)</t>
         </is>
       </c>
       <c r="D375" s="2" t="inlineStr">
         <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="E375" s="2" t="inlineStr"/>
-      <c r="F375" s="6" t="inlineStr">
-        <is>
-          <t>Added</t>
-        </is>
-      </c>
-      <c r="G375" s="2" t="inlineStr">
-        <is>
-          <t>MISSING: table had no PK</t>
-        </is>
-      </c>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="E375" s="2" t="inlineStr">
+        <is>
+          <t>Employee_Master.HRID</t>
+        </is>
+      </c>
+      <c r="F375" s="2" t="inlineStr">
+        <is>
+          <t>Kept</t>
+        </is>
+      </c>
+      <c r="G375" s="2" t="inlineStr"/>
     </row>
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
@@ -12186,30 +12171,26 @@
       </c>
       <c r="B376" s="2" t="inlineStr">
         <is>
-          <t>HRID</t>
+          <t>SSO_Id</t>
         </is>
       </c>
       <c r="C376" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(20)</t>
-        </is>
-      </c>
-      <c r="D376" s="2" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="E376" s="2" t="inlineStr">
-        <is>
-          <t>Employee_Master.HRID</t>
-        </is>
-      </c>
-      <c r="F376" s="2" t="inlineStr">
-        <is>
-          <t>Kept</t>
-        </is>
-      </c>
-      <c r="G376" s="2" t="inlineStr"/>
+          <t>VARCHAR(200)</t>
+        </is>
+      </c>
+      <c r="D376" s="2" t="inlineStr"/>
+      <c r="E376" s="2" t="inlineStr"/>
+      <c r="F376" s="5" t="inlineStr">
+        <is>
+          <t>Renamed</t>
+        </is>
+      </c>
+      <c r="G376" s="2" t="inlineStr">
+        <is>
+          <t>Was SSO</t>
+        </is>
+      </c>
     </row>
     <row r="377">
       <c r="A377" s="2" t="inlineStr">
@@ -12219,24 +12200,20 @@
       </c>
       <c r="B377" s="2" t="inlineStr">
         <is>
-          <t>SSO_Id</t>
-        </is>
-      </c>
-      <c r="C377" s="2" t="inlineStr">
-        <is>
-          <t>VARCHAR(200)</t>
-        </is>
-      </c>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="C377" s="2" t="inlineStr"/>
       <c r="D377" s="2" t="inlineStr"/>
       <c r="E377" s="2" t="inlineStr"/>
-      <c r="F377" s="5" t="inlineStr">
-        <is>
-          <t>Renamed</t>
+      <c r="F377" s="7" t="inlineStr">
+        <is>
+          <t>Removed</t>
         </is>
       </c>
       <c r="G377" s="2" t="inlineStr">
         <is>
-          <t>Was SSO</t>
+          <t>Duplicate of Employee_Master.Email</t>
         </is>
       </c>
     </row>
@@ -12248,20 +12225,24 @@
       </c>
       <c r="B378" s="2" t="inlineStr">
         <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="C378" s="2" t="inlineStr"/>
+          <t>Created_By</t>
+        </is>
+      </c>
+      <c r="C378" s="2" t="inlineStr">
+        <is>
+          <t>VARCHAR(100)</t>
+        </is>
+      </c>
       <c r="D378" s="2" t="inlineStr"/>
       <c r="E378" s="2" t="inlineStr"/>
-      <c r="F378" s="7" t="inlineStr">
-        <is>
-          <t>Removed</t>
+      <c r="F378" s="2" t="inlineStr">
+        <is>
+          <t>Kept</t>
         </is>
       </c>
       <c r="G378" s="2" t="inlineStr">
         <is>
-          <t>Duplicate of Employee_Master.Email</t>
+          <t>Audit column</t>
         </is>
       </c>
     </row>
@@ -12273,12 +12254,12 @@
       </c>
       <c r="B379" s="2" t="inlineStr">
         <is>
-          <t>Created_By</t>
+          <t>Created_Date</t>
         </is>
       </c>
       <c r="C379" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
+          <t>DATETIME2</t>
         </is>
       </c>
       <c r="D379" s="2" t="inlineStr"/>
@@ -12302,12 +12283,12 @@
       </c>
       <c r="B380" s="2" t="inlineStr">
         <is>
-          <t>Created_Date</t>
+          <t>Modified_By</t>
         </is>
       </c>
       <c r="C380" s="2" t="inlineStr">
         <is>
-          <t>DATETIME2</t>
+          <t>VARCHAR(100)</t>
         </is>
       </c>
       <c r="D380" s="2" t="inlineStr"/>
@@ -12331,12 +12312,12 @@
       </c>
       <c r="B381" s="2" t="inlineStr">
         <is>
-          <t>Modified_By</t>
+          <t>Modified_Date</t>
         </is>
       </c>
       <c r="C381" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(100)</t>
+          <t>DATETIME2</t>
         </is>
       </c>
       <c r="D381" s="2" t="inlineStr"/>
@@ -12355,29 +12336,33 @@
     <row r="382">
       <c r="A382" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_Login</t>
+          <t>ClearOps_UserLogin</t>
         </is>
       </c>
       <c r="B382" s="2" t="inlineStr">
         <is>
-          <t>Modified_Date</t>
+          <t>User_Login_Id</t>
         </is>
       </c>
       <c r="C382" s="2" t="inlineStr">
         <is>
-          <t>DATETIME2</t>
-        </is>
-      </c>
-      <c r="D382" s="2" t="inlineStr"/>
+          <t>BIGINT</t>
+        </is>
+      </c>
+      <c r="D382" s="2" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
       <c r="E382" s="2" t="inlineStr"/>
-      <c r="F382" s="2" t="inlineStr">
-        <is>
-          <t>Kept</t>
+      <c r="F382" s="6" t="inlineStr">
+        <is>
+          <t>Added</t>
         </is>
       </c>
       <c r="G382" s="2" t="inlineStr">
         <is>
-          <t>Audit column</t>
+          <t>MISSING: no PK</t>
         </is>
       </c>
     </row>
@@ -12389,7 +12374,7 @@
       </c>
       <c r="B383" s="2" t="inlineStr">
         <is>
-          <t>User_Login_Id</t>
+          <t>User_Id</t>
         </is>
       </c>
       <c r="C383" s="2" t="inlineStr">
@@ -12399,18 +12384,22 @@
       </c>
       <c r="D383" s="2" t="inlineStr">
         <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="E383" s="2" t="inlineStr"/>
-      <c r="F383" s="6" t="inlineStr">
-        <is>
-          <t>Added</t>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="E383" s="2" t="inlineStr">
+        <is>
+          <t>ClearOps_Users.User_Id</t>
+        </is>
+      </c>
+      <c r="F383" s="2" t="inlineStr">
+        <is>
+          <t>Kept</t>
         </is>
       </c>
       <c r="G383" s="2" t="inlineStr">
         <is>
-          <t>MISSING: no PK</t>
+          <t>Was userid</t>
         </is>
       </c>
     </row>
@@ -12422,32 +12411,24 @@
       </c>
       <c r="B384" s="2" t="inlineStr">
         <is>
-          <t>User_Id</t>
+          <t>Login_DateTime</t>
         </is>
       </c>
       <c r="C384" s="2" t="inlineStr">
         <is>
-          <t>BIGINT</t>
-        </is>
-      </c>
-      <c r="D384" s="2" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="E384" s="2" t="inlineStr">
-        <is>
-          <t>ClearOps_Users.User_Id</t>
-        </is>
-      </c>
-      <c r="F384" s="2" t="inlineStr">
-        <is>
-          <t>Kept</t>
+          <t>DATETIME2</t>
+        </is>
+      </c>
+      <c r="D384" s="2" t="inlineStr"/>
+      <c r="E384" s="2" t="inlineStr"/>
+      <c r="F384" s="5" t="inlineStr">
+        <is>
+          <t>Renamed</t>
         </is>
       </c>
       <c r="G384" s="2" t="inlineStr">
         <is>
-          <t>Was userid</t>
+          <t>Was logindatetimestampe (typo)</t>
         </is>
       </c>
     </row>
@@ -12459,26 +12440,22 @@
       </c>
       <c r="B385" s="2" t="inlineStr">
         <is>
-          <t>Login_DateTime</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="C385" s="2" t="inlineStr">
         <is>
-          <t>DATETIME2</t>
+          <t>VARCHAR(20)</t>
         </is>
       </c>
       <c r="D385" s="2" t="inlineStr"/>
       <c r="E385" s="2" t="inlineStr"/>
-      <c r="F385" s="5" t="inlineStr">
-        <is>
-          <t>Renamed</t>
-        </is>
-      </c>
-      <c r="G385" s="2" t="inlineStr">
-        <is>
-          <t>Was logindatetimestampe (typo)</t>
-        </is>
-      </c>
+      <c r="F385" s="2" t="inlineStr">
+        <is>
+          <t>Kept</t>
+        </is>
+      </c>
+      <c r="G385" s="2" t="inlineStr"/>
     </row>
     <row r="386">
       <c r="A386" s="2" t="inlineStr">
@@ -12488,32 +12465,32 @@
       </c>
       <c r="B386" s="2" t="inlineStr">
         <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="C386" s="2" t="inlineStr">
-        <is>
-          <t>VARCHAR(20)</t>
-        </is>
-      </c>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C386" s="2" t="inlineStr"/>
       <c r="D386" s="2" t="inlineStr"/>
       <c r="E386" s="2" t="inlineStr"/>
-      <c r="F386" s="2" t="inlineStr">
-        <is>
-          <t>Kept</t>
-        </is>
-      </c>
-      <c r="G386" s="2" t="inlineStr"/>
+      <c r="F386" s="7" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="G386" s="2" t="inlineStr">
+        <is>
+          <t>Duplicate of Employee_Master.Email</t>
+        </is>
+      </c>
     </row>
     <row r="387">
       <c r="A387" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_UserLogin</t>
+          <t>RolesandPermissions</t>
         </is>
       </c>
       <c r="B387" s="2" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>RoleName,RoleType,Module,Page_Id,Role_Access,AssignedUserCount,Status</t>
         </is>
       </c>
       <c r="C387" s="2" t="inlineStr"/>
@@ -12521,42 +12498,17 @@
       <c r="E387" s="2" t="inlineStr"/>
       <c r="F387" s="7" t="inlineStr">
         <is>
-          <t>Removed</t>
+          <t>Moved/Removed</t>
         </is>
       </c>
       <c r="G387" s="2" t="inlineStr">
         <is>
-          <t>Duplicate of Employee_Master.Email</t>
-        </is>
-      </c>
-    </row>
-    <row r="388">
-      <c r="A388" s="2" t="inlineStr">
-        <is>
-          <t>RolesandPermissions</t>
-        </is>
-      </c>
-      <c r="B388" s="2" t="inlineStr">
-        <is>
-          <t>RoleName,RoleType,Module,Page_Id,Role_Access,AssignedUserCount,Status</t>
-        </is>
-      </c>
-      <c r="C388" s="2" t="inlineStr"/>
-      <c r="D388" s="2" t="inlineStr"/>
-      <c r="E388" s="2" t="inlineStr"/>
-      <c r="F388" s="7" t="inlineStr">
-        <is>
-          <t>Moved/Removed</t>
-        </is>
-      </c>
-      <c r="G388" s="2" t="inlineStr">
-        <is>
           <t>Fully derivable from Role, Page, Permission, Access, Users (AssignedUserCount = COUNT)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G388"/>
+  <autoFilter ref="A1:G387"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -14350,7 +14302,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D82"/>
+  <dimension ref="A1:D81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -15594,22 +15546,22 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>ProjectManualCreation</t>
+          <t>Admin_IntegrationStatus</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>All columns</t>
-        </is>
-      </c>
-      <c r="C57" s="7" t="inlineStr">
-        <is>
-          <t>Moved/Removed</t>
+          <t>System_Name</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Renamed</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>Duplicate of Project_Master</t>
+          <t>Was System</t>
         </is>
       </c>
     </row>
@@ -15621,7 +15573,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>System_Name</t>
+          <t>Records_Captured</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
@@ -15631,19 +15583,19 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Was System</t>
+          <t>Was record_captured</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>Admin_IntegrationStatus</t>
+          <t>ClearOps_Logs</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Records_Captured</t>
+          <t>Cron_Job_Run_Id</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
@@ -15653,7 +15605,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>Was record_captured</t>
+          <t>Was cornjob run_id (typo)</t>
         </is>
       </c>
     </row>
@@ -15665,17 +15617,17 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Cron_Job_Run_Id</t>
-        </is>
-      </c>
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>Renamed</t>
+          <t>Run_Start</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>Added</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Was cornjob run_id (typo)</t>
+          <t>MISSING</t>
         </is>
       </c>
     </row>
@@ -15687,7 +15639,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Run_Start</t>
+          <t>Run_End</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -15709,7 +15661,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Run_End</t>
+          <t>Run_Status</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
@@ -15731,7 +15683,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Run_Status</t>
+          <t>Records_Processed</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
@@ -15753,7 +15705,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Records_Processed</t>
+          <t>Error_Message</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
@@ -15775,7 +15727,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Error_Message</t>
+          <t>Created_By</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -15785,7 +15737,7 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>Audit column (MISSING in sheet)</t>
         </is>
       </c>
     </row>
@@ -15797,7 +15749,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Created_By</t>
+          <t>Created_Date</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
@@ -15819,7 +15771,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Created_Date</t>
+          <t>Modified_By</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
@@ -15841,7 +15793,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Modified_By</t>
+          <t>Modified_Date</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -15858,12 +15810,12 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_Logs</t>
+          <t>ClearOps_Role</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Modified_Date</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -15873,19 +15825,19 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>Audit column (MISSING in sheet)</t>
+          <t>From RolesandPermissions</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_Role</t>
+          <t>ClearOps_Page</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Module</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -15895,73 +15847,73 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>From RolesandPermissions</t>
+          <t>Moved from RolesandPermissions</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_Page</t>
+          <t>ClearOps_Access</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Module</t>
-        </is>
-      </c>
-      <c r="C71" s="6" t="inlineStr">
-        <is>
-          <t>Added</t>
+          <t>Access_Type</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>Renamed</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>Moved from RolesandPermissions</t>
+          <t>Was Accrss_type (typo)</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_Access</t>
+          <t>ClearOps_Permission</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Access_Type</t>
-        </is>
-      </c>
-      <c r="C72" s="5" t="inlineStr">
-        <is>
-          <t>Renamed</t>
+          <t>HRID</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>Removed</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Was Accrss_type (typo)</t>
+          <t>A role permission is not per person; user-&gt;role is in ClearOps_Users</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_Permission</t>
+          <t>ClearOps_Users</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>HRID</t>
-        </is>
-      </c>
-      <c r="C73" s="7" t="inlineStr">
-        <is>
-          <t>Removed</t>
+          <t>User_Id</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>Renamed</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>A role permission is not per person; user-&gt;role is in ClearOps_Users</t>
+          <t>Was User_ID(PK) (sr_id)</t>
         </is>
       </c>
     </row>
@@ -15973,39 +15925,39 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>User_Id</t>
-        </is>
-      </c>
-      <c r="C74" s="5" t="inlineStr">
-        <is>
-          <t>Renamed</t>
+          <t>Role_Name, Name, Email</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>Removed</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Was User_ID(PK) (sr_id)</t>
+          <t>Derivable via Role_Id / HRID</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_Users</t>
+          <t>ClearOps_Login</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Role_Name, Name, Email</t>
-        </is>
-      </c>
-      <c r="C75" s="7" t="inlineStr">
-        <is>
-          <t>Removed</t>
+          <t>Login_Id</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>Added</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Derivable via Role_Id / HRID</t>
+          <t>MISSING: table had no PK</t>
         </is>
       </c>
     </row>
@@ -16017,17 +15969,17 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Login_Id</t>
-        </is>
-      </c>
-      <c r="C76" s="6" t="inlineStr">
-        <is>
-          <t>Added</t>
+          <t>SSO_Id</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>Renamed</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>MISSING: table had no PK</t>
+          <t>Was SSO</t>
         </is>
       </c>
     </row>
@@ -16039,39 +15991,39 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>SSO_Id</t>
-        </is>
-      </c>
-      <c r="C77" s="5" t="inlineStr">
-        <is>
-          <t>Renamed</t>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>Removed</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Was SSO</t>
+          <t>Duplicate of Employee_Master.Email</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_Login</t>
+          <t>ClearOps_UserLogin</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="C78" s="7" t="inlineStr">
-        <is>
-          <t>Removed</t>
+          <t>User_Login_Id</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>Added</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Duplicate of Employee_Master.Email</t>
+          <t>MISSING: no PK</t>
         </is>
       </c>
     </row>
@@ -16083,17 +16035,17 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>User_Login_Id</t>
-        </is>
-      </c>
-      <c r="C79" s="6" t="inlineStr">
-        <is>
-          <t>Added</t>
+          <t>Login_DateTime</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>Renamed</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>MISSING: no PK</t>
+          <t>Was logindatetimestampe (typo)</t>
         </is>
       </c>
     </row>
@@ -16105,66 +16057,44 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Login_DateTime</t>
-        </is>
-      </c>
-      <c r="C80" s="5" t="inlineStr">
-        <is>
-          <t>Renamed</t>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C80" s="7" t="inlineStr">
+        <is>
+          <t>Removed</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Was logindatetimestampe (typo)</t>
+          <t>Duplicate of Employee_Master.Email</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>ClearOps_UserLogin</t>
+          <t>RolesandPermissions</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>RoleName,RoleType,Module,Page_Id,Role_Access,AssignedUserCount,Status</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>Removed</t>
+          <t>Moved/Removed</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Duplicate of Employee_Master.Email</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="2" t="inlineStr">
-        <is>
-          <t>RolesandPermissions</t>
-        </is>
-      </c>
-      <c r="B82" s="2" t="inlineStr">
-        <is>
-          <t>RoleName,RoleType,Module,Page_Id,Role_Access,AssignedUserCount,Status</t>
-        </is>
-      </c>
-      <c r="C82" s="7" t="inlineStr">
-        <is>
-          <t>Moved/Removed</t>
-        </is>
-      </c>
-      <c r="D82" s="2" t="inlineStr">
-        <is>
           <t>Fully derivable from Role, Page, Permission, Access, Users (AssignedUserCount = COUNT)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D82"/>
+  <autoFilter ref="A1:D81"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Use the user's exact table names in mapping workbook
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A5mSLBPV7GuwkbXJCnEXu9
</commit_message>
<xml_diff>
--- a/ClearOps_Database_Mapped.xlsx
+++ b/ClearOps_Database_Mapped.xlsx
@@ -954,7 +954,7 @@
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>Time Off as ClearOps_TimeOff</t>
+          <t>Time Off as TimeOff(WD)</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
@@ -1185,7 +1185,7 @@
     <row r="29">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr">
@@ -1195,14 +1195,14 @@
       </c>
       <c r="C29" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS, Projects as Project_Master</t>
+          <t>Project Tasks (WBS) as ProjectWBS, Projects as Project_Master</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="15" t="inlineStr">
         <is>
-          <t>Project Estimates as ClearOps_ProjectEstimator</t>
+          <t>Project Estimates as Project_Estimator</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr">
@@ -1212,14 +1212,14 @@
       </c>
       <c r="C30" s="14" t="inlineStr">
         <is>
-          <t>Job Grades as Grades, Project Tasks (WBS) as ClearOps_ProjectWBS, Projects as Project_Master</t>
+          <t>Job Grades as Grades, Project Tasks (WBS) as ProjectWBS, Projects as Project_Master</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="15" t="inlineStr">
         <is>
-          <t>Project Finance Settings as ClearOps_ProjectSettings</t>
+          <t>Project Finance Settings as Project_Settings</t>
         </is>
       </c>
       <c r="B31" s="14" t="inlineStr">
@@ -1246,14 +1246,14 @@
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
-          <t>Currencies as ClearOps_Currency, Project Tasks (WBS) as ClearOps_ProjectWBS, Projects as Project_Master</t>
+          <t>Currencies as ClearOps_Currency, Project Tasks (WBS) as ProjectWBS, Projects as Project_Master</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="15" t="inlineStr">
         <is>
-          <t>Time Planner as ClearOps_ProjectTimePlanner</t>
+          <t>Time Planner as ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="C33" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS, Projects as Project_Master, Resources (bookable people) as Resources</t>
+          <t>Project Tasks (WBS) as ProjectWBS, Projects as Project_Master, Resources (bookable people) as Resources</t>
         </is>
       </c>
     </row>
@@ -1306,7 +1306,7 @@
       </c>
       <c r="C37" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS, Projects as Project_Master, Rate Card as ClearOps_RateCard, Resources (bookable people) as Resources</t>
+          <t>Project Tasks (WBS) as ProjectWBS, Projects as Project_Master, Rate Card as ClearOps_RateCard, Resources (bookable people) as Resources</t>
         </is>
       </c>
     </row>
@@ -1390,7 +1390,7 @@
     <row r="44">
       <c r="A44" s="15" t="inlineStr">
         <is>
-          <t>Access Levels as ClearOps_Access</t>
+          <t>Access Levels as ClearOpps_Access_table</t>
         </is>
       </c>
       <c r="B44" s="14" t="inlineStr">
@@ -1417,7 +1417,7 @@
       </c>
       <c r="C45" s="14" t="inlineStr">
         <is>
-          <t>Access Levels as ClearOps_Access, Pages as ClearOps_Page, Roles as ClearOps_Role</t>
+          <t>Access Levels as ClearOpps_Access_table, Pages as ClearOps_Page, Roles as ClearOps_Role</t>
         </is>
       </c>
     </row>
@@ -1441,7 +1441,7 @@
     <row r="47">
       <c r="A47" s="15" t="inlineStr">
         <is>
-          <t>Single Sign-On Link as ClearOps_Login</t>
+          <t>Single Sign-On Link as ClearOps_login</t>
         </is>
       </c>
       <c r="B47" s="14" t="inlineStr">
@@ -1458,7 +1458,7 @@
     <row r="48">
       <c r="A48" s="15" t="inlineStr">
         <is>
-          <t>Login History as ClearOps_UserLogin</t>
+          <t>Login History as UserLogin</t>
         </is>
       </c>
       <c r="B48" s="14" t="inlineStr">
@@ -1501,7 +1501,7 @@
     <row r="52">
       <c r="A52" s="15" t="inlineStr">
         <is>
-          <t>Integration Status as Admin_IntegrationStatus</t>
+          <t>Integration Status as Admin_Integration_Status</t>
         </is>
       </c>
       <c r="B52" s="14" t="inlineStr">
@@ -1518,7 +1518,7 @@
     <row r="53">
       <c r="A53" s="15" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="B53" s="14" t="inlineStr">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="C53" s="14" t="inlineStr">
         <is>
-          <t>Integration Status as Admin_IntegrationStatus</t>
+          <t>Integration Status as Admin_Integration_Status</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
     <row r="57">
       <c r="A57" s="17" t="inlineStr">
         <is>
-          <t>Project Forecasting (OLD) as ClearOps_ProjectForecasting</t>
+          <t>Project Forecasting (OLD) as Project_Forecasting</t>
         </is>
       </c>
       <c r="B57" s="14" t="inlineStr">
@@ -1578,7 +1578,7 @@
     <row r="58">
       <c r="A58" s="17" t="inlineStr">
         <is>
-          <t>Roles &amp; Permissions (OLD sheet) as RolesandPermissions</t>
+          <t>Roles &amp; Permissions (OLD sheet) as ClearOps_RolesandPermissions</t>
         </is>
       </c>
       <c r="B58" s="14" t="inlineStr">
@@ -2135,7 +2135,7 @@
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>Time Off as ClearOps_TimeOff</t>
+          <t>Time Off as TimeOff(WD)</t>
         </is>
       </c>
       <c r="C17" s="15" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>ClearOps_TimeOff</t>
+          <t>TimeOff(WD)</t>
         </is>
       </c>
       <c r="G17" s="14" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>Time Planner as ClearOps_ProjectTimePlanner</t>
+          <t>Time Planner as ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="C18" s="15" t="inlineStr">
@@ -2190,7 +2190,7 @@
       </c>
       <c r="F18" s="14" t="inlineStr">
         <is>
-          <t>ClearOps_ProjectTimePlanner</t>
+          <t>ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="G18" s="14" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="C20" s="15" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="F20" s="14" t="inlineStr">
         <is>
-          <t>ClearOps_ProjectWBS</t>
+          <t>ProjectWBS</t>
         </is>
       </c>
       <c r="G20" s="14" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>Project Estimates as ClearOps_ProjectEstimator</t>
+          <t>Project Estimates as Project_Estimator</t>
         </is>
       </c>
       <c r="C21" s="15" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="F21" s="14" t="inlineStr">
         <is>
-          <t>ClearOps_ProjectEstimator</t>
+          <t>Project_Estimator</t>
         </is>
       </c>
       <c r="G21" s="14" t="inlineStr">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>Project Finance Settings as ClearOps_ProjectSettings</t>
+          <t>Project Finance Settings as Project_Settings</t>
         </is>
       </c>
       <c r="C22" s="15" t="inlineStr">
@@ -2330,7 +2330,7 @@
       </c>
       <c r="F22" s="14" t="inlineStr">
         <is>
-          <t>ClearOps_ProjectSettings</t>
+          <t>Project_Settings</t>
         </is>
       </c>
       <c r="G22" s="14" t="inlineStr">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>Project Forecasting (OLD) as ClearOps_ProjectForecasting</t>
+          <t>Project Forecasting (OLD) as Project_Forecasting</t>
         </is>
       </c>
       <c r="C25" s="17" t="inlineStr">
@@ -2435,7 +2435,7 @@
       </c>
       <c r="F25" s="14" t="inlineStr">
         <is>
-          <t>ClearOps_ProjectForecasting</t>
+          <t>Project_Forecasting</t>
         </is>
       </c>
       <c r="G25" s="14" t="inlineStr">
@@ -2450,7 +2450,7 @@
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>Integration Status as Admin_IntegrationStatus</t>
+          <t>Integration Status as Admin_Integration_Status</t>
         </is>
       </c>
       <c r="C26" s="15" t="inlineStr">
@@ -2470,7 +2470,7 @@
       </c>
       <c r="F26" s="14" t="inlineStr">
         <is>
-          <t>Admin_IntegrationStatus</t>
+          <t>Admin_Integration_Status</t>
         </is>
       </c>
       <c r="G26" s="14" t="inlineStr">
@@ -2485,7 +2485,7 @@
       </c>
       <c r="B27" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="C27" s="15" t="inlineStr">
@@ -2505,7 +2505,7 @@
       </c>
       <c r="F27" s="14" t="inlineStr">
         <is>
-          <t>ClearOps_Logs</t>
+          <t>Logs_table</t>
         </is>
       </c>
       <c r="G27" s="14" t="inlineStr">
@@ -2590,7 +2590,7 @@
       </c>
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t>Access Levels as ClearOps_Access</t>
+          <t>Access Levels as ClearOpps_Access_table</t>
         </is>
       </c>
       <c r="C30" s="15" t="inlineStr">
@@ -2610,7 +2610,7 @@
       </c>
       <c r="F30" s="14" t="inlineStr">
         <is>
-          <t>ClearOps_Access</t>
+          <t>ClearOpps_Access_table</t>
         </is>
       </c>
       <c r="G30" s="14" t="inlineStr">
@@ -2695,7 +2695,7 @@
       </c>
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t>Single Sign-On Link as ClearOps_Login</t>
+          <t>Single Sign-On Link as ClearOps_login</t>
         </is>
       </c>
       <c r="C33" s="15" t="inlineStr">
@@ -2715,7 +2715,7 @@
       </c>
       <c r="F33" s="14" t="inlineStr">
         <is>
-          <t>ClearOps_Login</t>
+          <t>ClearOps_login</t>
         </is>
       </c>
       <c r="G33" s="14" t="inlineStr">
@@ -2730,7 +2730,7 @@
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>Login History as ClearOps_UserLogin</t>
+          <t>Login History as UserLogin</t>
         </is>
       </c>
       <c r="C34" s="15" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>ClearOps_UserLogin</t>
+          <t>UserLogin</t>
         </is>
       </c>
       <c r="G34" s="14" t="inlineStr">
@@ -2765,7 +2765,7 @@
       </c>
       <c r="B35" s="14" t="inlineStr">
         <is>
-          <t>Roles &amp; Permissions (OLD sheet) as RolesandPermissions</t>
+          <t>Roles &amp; Permissions (OLD sheet) as ClearOps_RolesandPermissions</t>
         </is>
       </c>
       <c r="C35" s="17" t="inlineStr">
@@ -2785,7 +2785,7 @@
       </c>
       <c r="F35" s="14" t="inlineStr">
         <is>
-          <t>RolesandPermissions</t>
+          <t>ClearOps_RolesandPermissions</t>
         </is>
       </c>
       <c r="G35" s="14" t="inlineStr">
@@ -6336,7 +6336,7 @@
       </c>
       <c r="G118" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
     </row>
@@ -7662,7 +7662,7 @@
     <row r="162">
       <c r="A162" s="14" t="inlineStr">
         <is>
-          <t>Time Off as ClearOps_TimeOff</t>
+          <t>Time Off as TimeOff(WD)</t>
         </is>
       </c>
       <c r="B162" s="14" t="inlineStr">
@@ -7682,7 +7682,7 @@
       </c>
       <c r="E162" s="14" t="inlineStr">
         <is>
-          <t>Unique number of each row in Time Off as ClearOps_TimeOff</t>
+          <t>Unique number of each row in Time Off as TimeOff(WD)</t>
         </is>
       </c>
       <c r="F162" s="14" t="inlineStr">
@@ -7695,7 +7695,7 @@
     <row r="163">
       <c r="A163" s="14" t="inlineStr">
         <is>
-          <t>Time Off as ClearOps_TimeOff</t>
+          <t>Time Off as TimeOff(WD)</t>
         </is>
       </c>
       <c r="B163" s="14" t="inlineStr">
@@ -7732,7 +7732,7 @@
     <row r="164">
       <c r="A164" s="14" t="inlineStr">
         <is>
-          <t>Time Off as ClearOps_TimeOff</t>
+          <t>Time Off as TimeOff(WD)</t>
         </is>
       </c>
       <c r="B164" s="14" t="inlineStr">
@@ -7761,7 +7761,7 @@
     <row r="165">
       <c r="A165" s="14" t="inlineStr">
         <is>
-          <t>Time Off as ClearOps_TimeOff</t>
+          <t>Time Off as TimeOff(WD)</t>
         </is>
       </c>
       <c r="B165" s="16" t="inlineStr">
@@ -7790,7 +7790,7 @@
     <row r="166">
       <c r="A166" s="14" t="inlineStr">
         <is>
-          <t>Time Off as ClearOps_TimeOff</t>
+          <t>Time Off as TimeOff(WD)</t>
         </is>
       </c>
       <c r="B166" s="16" t="inlineStr">
@@ -7819,7 +7819,7 @@
     <row r="167">
       <c r="A167" s="14" t="inlineStr">
         <is>
-          <t>Time Off as ClearOps_TimeOff</t>
+          <t>Time Off as TimeOff(WD)</t>
         </is>
       </c>
       <c r="B167" s="14" t="inlineStr">
@@ -7848,7 +7848,7 @@
     <row r="168">
       <c r="A168" s="14" t="inlineStr">
         <is>
-          <t>Time Off as ClearOps_TimeOff</t>
+          <t>Time Off as TimeOff(WD)</t>
         </is>
       </c>
       <c r="B168" s="14" t="inlineStr">
@@ -7877,7 +7877,7 @@
     <row r="169">
       <c r="A169" s="14" t="inlineStr">
         <is>
-          <t>Time Off as ClearOps_TimeOff</t>
+          <t>Time Off as TimeOff(WD)</t>
         </is>
       </c>
       <c r="B169" s="14" t="inlineStr">
@@ -7906,7 +7906,7 @@
     <row r="170">
       <c r="A170" s="14" t="inlineStr">
         <is>
-          <t>Time Off as ClearOps_TimeOff</t>
+          <t>Time Off as TimeOff(WD)</t>
         </is>
       </c>
       <c r="B170" s="14" t="inlineStr">
@@ -7935,7 +7935,7 @@
     <row r="171">
       <c r="A171" s="14" t="inlineStr">
         <is>
-          <t>Time Planner as ClearOps_ProjectTimePlanner</t>
+          <t>Time Planner as ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="B171" s="15" t="inlineStr">
@@ -7955,7 +7955,7 @@
       </c>
       <c r="E171" s="14" t="inlineStr">
         <is>
-          <t>Unique number of each row in Time Planner as ClearOps_ProjectTimePlanner [Was Project_Time_Panner_id (typo)]</t>
+          <t>Unique number of each row in Time Planner as ClearOps_Project_Time_Planner [Was Project_Time_Panner_id (typo)]</t>
         </is>
       </c>
       <c r="F171" s="14" t="inlineStr">
@@ -7968,7 +7968,7 @@
     <row r="172">
       <c r="A172" s="14" t="inlineStr">
         <is>
-          <t>Time Planner as ClearOps_ProjectTimePlanner</t>
+          <t>Time Planner as ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="B172" s="16" t="inlineStr">
@@ -8005,7 +8005,7 @@
     <row r="173">
       <c r="A173" s="14" t="inlineStr">
         <is>
-          <t>Time Planner as ClearOps_ProjectTimePlanner</t>
+          <t>Time Planner as ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="B173" s="14" t="inlineStr">
@@ -8035,14 +8035,14 @@
       </c>
       <c r="G173" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="14" t="inlineStr">
         <is>
-          <t>Time Planner as ClearOps_ProjectTimePlanner</t>
+          <t>Time Planner as ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="B174" s="14" t="inlineStr">
@@ -8079,7 +8079,7 @@
     <row r="175">
       <c r="A175" s="14" t="inlineStr">
         <is>
-          <t>Time Planner as ClearOps_ProjectTimePlanner</t>
+          <t>Time Planner as ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="B175" s="14" t="inlineStr">
@@ -8108,7 +8108,7 @@
     <row r="176">
       <c r="A176" s="14" t="inlineStr">
         <is>
-          <t>Time Planner as ClearOps_ProjectTimePlanner</t>
+          <t>Time Planner as ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="B176" s="14" t="inlineStr">
@@ -8137,7 +8137,7 @@
     <row r="177">
       <c r="A177" s="14" t="inlineStr">
         <is>
-          <t>Time Planner as ClearOps_ProjectTimePlanner</t>
+          <t>Time Planner as ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="B177" s="14" t="inlineStr">
@@ -8166,7 +8166,7 @@
     <row r="178">
       <c r="A178" s="14" t="inlineStr">
         <is>
-          <t>Time Planner as ClearOps_ProjectTimePlanner</t>
+          <t>Time Planner as ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="B178" s="14" t="inlineStr">
@@ -8195,7 +8195,7 @@
     <row r="179">
       <c r="A179" s="14" t="inlineStr">
         <is>
-          <t>Time Planner as ClearOps_ProjectTimePlanner</t>
+          <t>Time Planner as ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="B179" s="14" t="inlineStr">
@@ -8224,7 +8224,7 @@
     <row r="180">
       <c r="A180" s="14" t="inlineStr">
         <is>
-          <t>Time Planner as ClearOps_ProjectTimePlanner</t>
+          <t>Time Planner as ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="B180" s="14" t="inlineStr">
@@ -8253,7 +8253,7 @@
     <row r="181">
       <c r="A181" s="14" t="inlineStr">
         <is>
-          <t>Time Planner as ClearOps_ProjectTimePlanner</t>
+          <t>Time Planner as ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="B181" s="14" t="inlineStr">
@@ -8282,7 +8282,7 @@
     <row r="182">
       <c r="A182" s="14" t="inlineStr">
         <is>
-          <t>Time Planner as ClearOps_ProjectTimePlanner</t>
+          <t>Time Planner as ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="B182" s="14" t="inlineStr">
@@ -8311,7 +8311,7 @@
     <row r="183">
       <c r="A183" s="14" t="inlineStr">
         <is>
-          <t>Time Planner as ClearOps_ProjectTimePlanner</t>
+          <t>Time Planner as ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="B183" s="14" t="inlineStr">
@@ -8340,7 +8340,7 @@
     <row r="184">
       <c r="A184" s="14" t="inlineStr">
         <is>
-          <t>Time Planner as ClearOps_ProjectTimePlanner</t>
+          <t>Time Planner as ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="B184" s="14" t="inlineStr">
@@ -8369,7 +8369,7 @@
     <row r="185">
       <c r="A185" s="14" t="inlineStr">
         <is>
-          <t>Time Planner as ClearOps_ProjectTimePlanner</t>
+          <t>Time Planner as ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="B185" s="14" t="inlineStr">
@@ -8398,7 +8398,7 @@
     <row r="186">
       <c r="A186" s="14" t="inlineStr">
         <is>
-          <t>Time Planner as ClearOps_ProjectTimePlanner</t>
+          <t>Time Planner as ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="B186" s="14" t="inlineStr">
@@ -9526,7 +9526,7 @@
     <row r="222">
       <c r="A222" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B222" s="15" t="inlineStr">
@@ -9559,7 +9559,7 @@
     <row r="223">
       <c r="A223" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B223" s="14" t="inlineStr">
@@ -9596,7 +9596,7 @@
     <row r="224">
       <c r="A224" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B224" s="15" t="inlineStr">
@@ -9626,14 +9626,14 @@
       </c>
       <c r="G224" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B225" s="14" t="inlineStr">
@@ -9663,14 +9663,14 @@
       </c>
       <c r="G225" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B226" s="14" t="inlineStr">
@@ -9699,7 +9699,7 @@
     <row r="227">
       <c r="A227" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B227" s="16" t="inlineStr">
@@ -9728,7 +9728,7 @@
     <row r="228">
       <c r="A228" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B228" s="15" t="inlineStr">
@@ -9757,7 +9757,7 @@
     <row r="229">
       <c r="A229" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B229" s="14" t="inlineStr">
@@ -9786,7 +9786,7 @@
     <row r="230">
       <c r="A230" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B230" s="14" t="inlineStr">
@@ -9815,7 +9815,7 @@
     <row r="231">
       <c r="A231" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B231" s="14" t="inlineStr">
@@ -9844,7 +9844,7 @@
     <row r="232">
       <c r="A232" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B232" s="14" t="inlineStr">
@@ -9873,7 +9873,7 @@
     <row r="233">
       <c r="A233" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B233" s="14" t="inlineStr">
@@ -9902,7 +9902,7 @@
     <row r="234">
       <c r="A234" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B234" s="14" t="inlineStr">
@@ -9931,7 +9931,7 @@
     <row r="235">
       <c r="A235" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B235" s="14" t="inlineStr">
@@ -9960,7 +9960,7 @@
     <row r="236">
       <c r="A236" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B236" s="15" t="inlineStr">
@@ -9989,7 +9989,7 @@
     <row r="237">
       <c r="A237" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B237" s="15" t="inlineStr">
@@ -10018,7 +10018,7 @@
     <row r="238">
       <c r="A238" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B238" s="14" t="inlineStr">
@@ -10047,7 +10047,7 @@
     <row r="239">
       <c r="A239" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B239" s="14" t="inlineStr">
@@ -10076,7 +10076,7 @@
     <row r="240">
       <c r="A240" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B240" s="14" t="inlineStr">
@@ -10105,7 +10105,7 @@
     <row r="241">
       <c r="A241" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B241" s="14" t="inlineStr">
@@ -10134,7 +10134,7 @@
     <row r="242">
       <c r="A242" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B242" s="14" t="inlineStr">
@@ -10163,7 +10163,7 @@
     <row r="243">
       <c r="A243" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B243" s="14" t="inlineStr">
@@ -10192,7 +10192,7 @@
     <row r="244">
       <c r="A244" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B244" s="14" t="inlineStr">
@@ -10221,7 +10221,7 @@
     <row r="245">
       <c r="A245" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B245" s="14" t="inlineStr">
@@ -10250,7 +10250,7 @@
     <row r="246">
       <c r="A246" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B246" s="14" t="inlineStr">
@@ -10279,7 +10279,7 @@
     <row r="247">
       <c r="A247" s="14" t="inlineStr">
         <is>
-          <t>Project Estimates as ClearOps_ProjectEstimator</t>
+          <t>Project Estimates as Project_Estimator</t>
         </is>
       </c>
       <c r="B247" s="15" t="inlineStr">
@@ -10312,7 +10312,7 @@
     <row r="248">
       <c r="A248" s="14" t="inlineStr">
         <is>
-          <t>Project Estimates as ClearOps_ProjectEstimator</t>
+          <t>Project Estimates as Project_Estimator</t>
         </is>
       </c>
       <c r="B248" s="14" t="inlineStr">
@@ -10349,7 +10349,7 @@
     <row r="249">
       <c r="A249" s="14" t="inlineStr">
         <is>
-          <t>Project Estimates as ClearOps_ProjectEstimator</t>
+          <t>Project Estimates as Project_Estimator</t>
         </is>
       </c>
       <c r="B249" s="14" t="inlineStr">
@@ -10379,14 +10379,14 @@
       </c>
       <c r="G249" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="14" t="inlineStr">
         <is>
-          <t>Project Estimates as ClearOps_ProjectEstimator</t>
+          <t>Project Estimates as Project_Estimator</t>
         </is>
       </c>
       <c r="B250" s="15" t="inlineStr">
@@ -10423,7 +10423,7 @@
     <row r="251">
       <c r="A251" s="14" t="inlineStr">
         <is>
-          <t>Project Estimates as ClearOps_ProjectEstimator</t>
+          <t>Project Estimates as Project_Estimator</t>
         </is>
       </c>
       <c r="B251" s="14" t="inlineStr">
@@ -10452,7 +10452,7 @@
     <row r="252">
       <c r="A252" s="14" t="inlineStr">
         <is>
-          <t>Project Estimates as ClearOps_ProjectEstimator</t>
+          <t>Project Estimates as Project_Estimator</t>
         </is>
       </c>
       <c r="B252" s="14" t="inlineStr">
@@ -10481,7 +10481,7 @@
     <row r="253">
       <c r="A253" s="14" t="inlineStr">
         <is>
-          <t>Project Estimates as ClearOps_ProjectEstimator</t>
+          <t>Project Estimates as Project_Estimator</t>
         </is>
       </c>
       <c r="B253" s="14" t="inlineStr">
@@ -10510,7 +10510,7 @@
     <row r="254">
       <c r="A254" s="14" t="inlineStr">
         <is>
-          <t>Project Estimates as ClearOps_ProjectEstimator</t>
+          <t>Project Estimates as Project_Estimator</t>
         </is>
       </c>
       <c r="B254" s="14" t="inlineStr">
@@ -10539,7 +10539,7 @@
     <row r="255">
       <c r="A255" s="14" t="inlineStr">
         <is>
-          <t>Project Estimates as ClearOps_ProjectEstimator</t>
+          <t>Project Estimates as Project_Estimator</t>
         </is>
       </c>
       <c r="B255" s="14" t="inlineStr">
@@ -10568,7 +10568,7 @@
     <row r="256">
       <c r="A256" s="14" t="inlineStr">
         <is>
-          <t>Project Estimates as ClearOps_ProjectEstimator</t>
+          <t>Project Estimates as Project_Estimator</t>
         </is>
       </c>
       <c r="B256" s="14" t="inlineStr">
@@ -10597,7 +10597,7 @@
     <row r="257">
       <c r="A257" s="14" t="inlineStr">
         <is>
-          <t>Project Estimates as ClearOps_ProjectEstimator</t>
+          <t>Project Estimates as Project_Estimator</t>
         </is>
       </c>
       <c r="B257" s="14" t="inlineStr">
@@ -10626,7 +10626,7 @@
     <row r="258">
       <c r="A258" s="14" t="inlineStr">
         <is>
-          <t>Project Estimates as ClearOps_ProjectEstimator</t>
+          <t>Project Estimates as Project_Estimator</t>
         </is>
       </c>
       <c r="B258" s="14" t="inlineStr">
@@ -10655,7 +10655,7 @@
     <row r="259">
       <c r="A259" s="14" t="inlineStr">
         <is>
-          <t>Project Estimates as ClearOps_ProjectEstimator</t>
+          <t>Project Estimates as Project_Estimator</t>
         </is>
       </c>
       <c r="B259" s="14" t="inlineStr">
@@ -10684,7 +10684,7 @@
     <row r="260">
       <c r="A260" s="14" t="inlineStr">
         <is>
-          <t>Project Estimates as ClearOps_ProjectEstimator</t>
+          <t>Project Estimates as Project_Estimator</t>
         </is>
       </c>
       <c r="B260" s="14" t="inlineStr">
@@ -10713,7 +10713,7 @@
     <row r="261">
       <c r="A261" s="14" t="inlineStr">
         <is>
-          <t>Project Finance Settings as ClearOps_ProjectSettings</t>
+          <t>Project Finance Settings as Project_Settings</t>
         </is>
       </c>
       <c r="B261" s="14" t="inlineStr">
@@ -10733,7 +10733,7 @@
       </c>
       <c r="E261" s="14" t="inlineStr">
         <is>
-          <t>Unique number of each row in Project Finance Settings as ClearOps_ProjectSettings</t>
+          <t>Unique number of each row in Project Finance Settings as Project_Settings</t>
         </is>
       </c>
       <c r="F261" s="14" t="inlineStr">
@@ -10746,7 +10746,7 @@
     <row r="262">
       <c r="A262" s="14" t="inlineStr">
         <is>
-          <t>Project Finance Settings as ClearOps_ProjectSettings</t>
+          <t>Project Finance Settings as Project_Settings</t>
         </is>
       </c>
       <c r="B262" s="14" t="inlineStr">
@@ -10783,7 +10783,7 @@
     <row r="263">
       <c r="A263" s="14" t="inlineStr">
         <is>
-          <t>Project Finance Settings as ClearOps_ProjectSettings</t>
+          <t>Project Finance Settings as Project_Settings</t>
         </is>
       </c>
       <c r="B263" s="14" t="inlineStr">
@@ -10812,7 +10812,7 @@
     <row r="264">
       <c r="A264" s="14" t="inlineStr">
         <is>
-          <t>Project Finance Settings as ClearOps_ProjectSettings</t>
+          <t>Project Finance Settings as Project_Settings</t>
         </is>
       </c>
       <c r="B264" s="14" t="inlineStr">
@@ -10841,7 +10841,7 @@
     <row r="265">
       <c r="A265" s="14" t="inlineStr">
         <is>
-          <t>Project Finance Settings as ClearOps_ProjectSettings</t>
+          <t>Project Finance Settings as Project_Settings</t>
         </is>
       </c>
       <c r="B265" s="14" t="inlineStr">
@@ -10870,7 +10870,7 @@
     <row r="266">
       <c r="A266" s="14" t="inlineStr">
         <is>
-          <t>Project Finance Settings as ClearOps_ProjectSettings</t>
+          <t>Project Finance Settings as Project_Settings</t>
         </is>
       </c>
       <c r="B266" s="14" t="inlineStr">
@@ -10899,7 +10899,7 @@
     <row r="267">
       <c r="A267" s="14" t="inlineStr">
         <is>
-          <t>Project Finance Settings as ClearOps_ProjectSettings</t>
+          <t>Project Finance Settings as Project_Settings</t>
         </is>
       </c>
       <c r="B267" s="14" t="inlineStr">
@@ -10928,7 +10928,7 @@
     <row r="268">
       <c r="A268" s="14" t="inlineStr">
         <is>
-          <t>Project Finance Settings as ClearOps_ProjectSettings</t>
+          <t>Project Finance Settings as Project_Settings</t>
         </is>
       </c>
       <c r="B268" s="14" t="inlineStr">
@@ -10957,7 +10957,7 @@
     <row r="269">
       <c r="A269" s="14" t="inlineStr">
         <is>
-          <t>Project Finance Settings as ClearOps_ProjectSettings</t>
+          <t>Project Finance Settings as Project_Settings</t>
         </is>
       </c>
       <c r="B269" s="14" t="inlineStr">
@@ -10986,7 +10986,7 @@
     <row r="270">
       <c r="A270" s="14" t="inlineStr">
         <is>
-          <t>Project Finance Settings as ClearOps_ProjectSettings</t>
+          <t>Project Finance Settings as Project_Settings</t>
         </is>
       </c>
       <c r="B270" s="14" t="inlineStr">
@@ -11015,7 +11015,7 @@
     <row r="271">
       <c r="A271" s="14" t="inlineStr">
         <is>
-          <t>Project Finance Settings as ClearOps_ProjectSettings</t>
+          <t>Project Finance Settings as Project_Settings</t>
         </is>
       </c>
       <c r="B271" s="14" t="inlineStr">
@@ -11044,7 +11044,7 @@
     <row r="272">
       <c r="A272" s="14" t="inlineStr">
         <is>
-          <t>Project Finance Settings as ClearOps_ProjectSettings</t>
+          <t>Project Finance Settings as Project_Settings</t>
         </is>
       </c>
       <c r="B272" s="14" t="inlineStr">
@@ -11073,7 +11073,7 @@
     <row r="273">
       <c r="A273" s="14" t="inlineStr">
         <is>
-          <t>Project Finance Settings as ClearOps_ProjectSettings</t>
+          <t>Project Finance Settings as Project_Settings</t>
         </is>
       </c>
       <c r="B273" s="14" t="inlineStr">
@@ -11102,7 +11102,7 @@
     <row r="274">
       <c r="A274" s="14" t="inlineStr">
         <is>
-          <t>Project Finance Settings as ClearOps_ProjectSettings</t>
+          <t>Project Finance Settings as Project_Settings</t>
         </is>
       </c>
       <c r="B274" s="14" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="G277" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
     </row>
@@ -11817,7 +11817,7 @@
     <row r="297">
       <c r="A297" s="14" t="inlineStr">
         <is>
-          <t>Integration Status as Admin_IntegrationStatus</t>
+          <t>Integration Status as Admin_Integration_Status</t>
         </is>
       </c>
       <c r="B297" s="14" t="inlineStr">
@@ -11850,7 +11850,7 @@
     <row r="298">
       <c r="A298" s="14" t="inlineStr">
         <is>
-          <t>Integration Status as Admin_IntegrationStatus</t>
+          <t>Integration Status as Admin_Integration_Status</t>
         </is>
       </c>
       <c r="B298" s="15" t="inlineStr">
@@ -11879,7 +11879,7 @@
     <row r="299">
       <c r="A299" s="14" t="inlineStr">
         <is>
-          <t>Integration Status as Admin_IntegrationStatus</t>
+          <t>Integration Status as Admin_Integration_Status</t>
         </is>
       </c>
       <c r="B299" s="14" t="inlineStr">
@@ -11908,7 +11908,7 @@
     <row r="300">
       <c r="A300" s="14" t="inlineStr">
         <is>
-          <t>Integration Status as Admin_IntegrationStatus</t>
+          <t>Integration Status as Admin_Integration_Status</t>
         </is>
       </c>
       <c r="B300" s="14" t="inlineStr">
@@ -11937,7 +11937,7 @@
     <row r="301">
       <c r="A301" s="14" t="inlineStr">
         <is>
-          <t>Integration Status as Admin_IntegrationStatus</t>
+          <t>Integration Status as Admin_Integration_Status</t>
         </is>
       </c>
       <c r="B301" s="15" t="inlineStr">
@@ -11966,7 +11966,7 @@
     <row r="302">
       <c r="A302" s="14" t="inlineStr">
         <is>
-          <t>Integration Status as Admin_IntegrationStatus</t>
+          <t>Integration Status as Admin_Integration_Status</t>
         </is>
       </c>
       <c r="B302" s="14" t="inlineStr">
@@ -11995,7 +11995,7 @@
     <row r="303">
       <c r="A303" s="14" t="inlineStr">
         <is>
-          <t>Integration Status as Admin_IntegrationStatus</t>
+          <t>Integration Status as Admin_Integration_Status</t>
         </is>
       </c>
       <c r="B303" s="14" t="inlineStr">
@@ -12024,7 +12024,7 @@
     <row r="304">
       <c r="A304" s="14" t="inlineStr">
         <is>
-          <t>Integration Status as Admin_IntegrationStatus</t>
+          <t>Integration Status as Admin_Integration_Status</t>
         </is>
       </c>
       <c r="B304" s="14" t="inlineStr">
@@ -12053,7 +12053,7 @@
     <row r="305">
       <c r="A305" s="14" t="inlineStr">
         <is>
-          <t>Integration Status as Admin_IntegrationStatus</t>
+          <t>Integration Status as Admin_Integration_Status</t>
         </is>
       </c>
       <c r="B305" s="14" t="inlineStr">
@@ -12082,7 +12082,7 @@
     <row r="306">
       <c r="A306" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="B306" s="14" t="inlineStr">
@@ -12102,7 +12102,7 @@
       </c>
       <c r="E306" s="14" t="inlineStr">
         <is>
-          <t>Unique number of each row in Integration Run Log as ClearOps_Logs</t>
+          <t>Unique number of each row in Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="F306" s="14" t="inlineStr">
@@ -12115,7 +12115,7 @@
     <row r="307">
       <c r="A307" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="B307" s="14" t="inlineStr">
@@ -12145,14 +12145,14 @@
       </c>
       <c r="G307" s="14" t="inlineStr">
         <is>
-          <t>Integration Status as Admin_IntegrationStatus</t>
+          <t>Integration Status as Admin_Integration_Status</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="B308" s="15" t="inlineStr">
@@ -12181,7 +12181,7 @@
     <row r="309">
       <c r="A309" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="B309" s="16" t="inlineStr">
@@ -12210,7 +12210,7 @@
     <row r="310">
       <c r="A310" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="B310" s="16" t="inlineStr">
@@ -12239,7 +12239,7 @@
     <row r="311">
       <c r="A311" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="B311" s="16" t="inlineStr">
@@ -12268,7 +12268,7 @@
     <row r="312">
       <c r="A312" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="B312" s="16" t="inlineStr">
@@ -12297,7 +12297,7 @@
     <row r="313">
       <c r="A313" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="B313" s="16" t="inlineStr">
@@ -12326,7 +12326,7 @@
     <row r="314">
       <c r="A314" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="B314" s="16" t="inlineStr">
@@ -12355,7 +12355,7 @@
     <row r="315">
       <c r="A315" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="B315" s="16" t="inlineStr">
@@ -12384,7 +12384,7 @@
     <row r="316">
       <c r="A316" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="B316" s="16" t="inlineStr">
@@ -12413,7 +12413,7 @@
     <row r="317">
       <c r="A317" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="B317" s="16" t="inlineStr">
@@ -12549,7 +12549,7 @@
       <c r="D321" s="14" t="inlineStr"/>
       <c r="E321" s="14" t="inlineStr">
         <is>
-          <t>Active or inactive [From RolesandPermissions]</t>
+          <t>Active or inactive [From ClearOps_RolesandPermissions]</t>
         </is>
       </c>
       <c r="F321" s="14" t="inlineStr">
@@ -12785,7 +12785,7 @@
       <c r="D329" s="14" t="inlineStr"/>
       <c r="E329" s="14" t="inlineStr">
         <is>
-          <t>Group of pages [Moved from RolesandPermissions]</t>
+          <t>Group of pages [Moved from ClearOps_RolesandPermissions]</t>
         </is>
       </c>
       <c r="F329" s="14" t="inlineStr">
@@ -12914,7 +12914,7 @@
     <row r="334">
       <c r="A334" s="14" t="inlineStr">
         <is>
-          <t>Access Levels as ClearOps_Access</t>
+          <t>Access Levels as ClearOpps_Access_table</t>
         </is>
       </c>
       <c r="B334" s="14" t="inlineStr">
@@ -12947,7 +12947,7 @@
     <row r="335">
       <c r="A335" s="14" t="inlineStr">
         <is>
-          <t>Access Levels as ClearOps_Access</t>
+          <t>Access Levels as ClearOpps_Access_table</t>
         </is>
       </c>
       <c r="B335" s="15" t="inlineStr">
@@ -12976,7 +12976,7 @@
     <row r="336">
       <c r="A336" s="14" t="inlineStr">
         <is>
-          <t>Access Levels as ClearOps_Access</t>
+          <t>Access Levels as ClearOpps_Access_table</t>
         </is>
       </c>
       <c r="B336" s="14" t="inlineStr">
@@ -13005,7 +13005,7 @@
     <row r="337">
       <c r="A337" s="14" t="inlineStr">
         <is>
-          <t>Access Levels as ClearOps_Access</t>
+          <t>Access Levels as ClearOpps_Access_table</t>
         </is>
       </c>
       <c r="B337" s="14" t="inlineStr">
@@ -13034,7 +13034,7 @@
     <row r="338">
       <c r="A338" s="14" t="inlineStr">
         <is>
-          <t>Access Levels as ClearOps_Access</t>
+          <t>Access Levels as ClearOpps_Access_table</t>
         </is>
       </c>
       <c r="B338" s="14" t="inlineStr">
@@ -13063,7 +13063,7 @@
     <row r="339">
       <c r="A339" s="14" t="inlineStr">
         <is>
-          <t>Access Levels as ClearOps_Access</t>
+          <t>Access Levels as ClearOpps_Access_table</t>
         </is>
       </c>
       <c r="B339" s="14" t="inlineStr">
@@ -13229,7 +13229,7 @@
       </c>
       <c r="G343" s="14" t="inlineStr">
         <is>
-          <t>Access Levels as ClearOps_Access</t>
+          <t>Access Levels as ClearOpps_Access_table</t>
         </is>
       </c>
     </row>
@@ -13604,7 +13604,7 @@
     <row r="356">
       <c r="A356" s="14" t="inlineStr">
         <is>
-          <t>Single Sign-On Link as ClearOps_Login</t>
+          <t>Single Sign-On Link as ClearOps_login</t>
         </is>
       </c>
       <c r="B356" s="16" t="inlineStr">
@@ -13624,7 +13624,7 @@
       </c>
       <c r="E356" s="14" t="inlineStr">
         <is>
-          <t>Unique number of each row in Single Sign-On Link as ClearOps_Login [Was missing – table had no PK]</t>
+          <t>Unique number of each row in Single Sign-On Link as ClearOps_login [Was missing – table had no PK]</t>
         </is>
       </c>
       <c r="F356" s="14" t="inlineStr">
@@ -13637,7 +13637,7 @@
     <row r="357">
       <c r="A357" s="14" t="inlineStr">
         <is>
-          <t>Single Sign-On Link as ClearOps_Login</t>
+          <t>Single Sign-On Link as ClearOps_login</t>
         </is>
       </c>
       <c r="B357" s="14" t="inlineStr">
@@ -13674,7 +13674,7 @@
     <row r="358">
       <c r="A358" s="14" t="inlineStr">
         <is>
-          <t>Single Sign-On Link as ClearOps_Login</t>
+          <t>Single Sign-On Link as ClearOps_login</t>
         </is>
       </c>
       <c r="B358" s="15" t="inlineStr">
@@ -13703,7 +13703,7 @@
     <row r="359">
       <c r="A359" s="14" t="inlineStr">
         <is>
-          <t>Single Sign-On Link as ClearOps_Login</t>
+          <t>Single Sign-On Link as ClearOps_login</t>
         </is>
       </c>
       <c r="B359" s="14" t="inlineStr">
@@ -13732,7 +13732,7 @@
     <row r="360">
       <c r="A360" s="14" t="inlineStr">
         <is>
-          <t>Single Sign-On Link as ClearOps_Login</t>
+          <t>Single Sign-On Link as ClearOps_login</t>
         </is>
       </c>
       <c r="B360" s="14" t="inlineStr">
@@ -13761,7 +13761,7 @@
     <row r="361">
       <c r="A361" s="14" t="inlineStr">
         <is>
-          <t>Single Sign-On Link as ClearOps_Login</t>
+          <t>Single Sign-On Link as ClearOps_login</t>
         </is>
       </c>
       <c r="B361" s="14" t="inlineStr">
@@ -13790,7 +13790,7 @@
     <row r="362">
       <c r="A362" s="14" t="inlineStr">
         <is>
-          <t>Single Sign-On Link as ClearOps_Login</t>
+          <t>Single Sign-On Link as ClearOps_login</t>
         </is>
       </c>
       <c r="B362" s="14" t="inlineStr">
@@ -13819,7 +13819,7 @@
     <row r="363">
       <c r="A363" s="14" t="inlineStr">
         <is>
-          <t>Login History as ClearOps_UserLogin</t>
+          <t>Login History as UserLogin</t>
         </is>
       </c>
       <c r="B363" s="16" t="inlineStr">
@@ -13839,7 +13839,7 @@
       </c>
       <c r="E363" s="14" t="inlineStr">
         <is>
-          <t>Unique number of each row in Login History as ClearOps_UserLogin [Was missing – no PK]</t>
+          <t>Unique number of each row in Login History as UserLogin [Was missing – no PK]</t>
         </is>
       </c>
       <c r="F363" s="14" t="inlineStr">
@@ -13852,7 +13852,7 @@
     <row r="364">
       <c r="A364" s="14" t="inlineStr">
         <is>
-          <t>Login History as ClearOps_UserLogin</t>
+          <t>Login History as UserLogin</t>
         </is>
       </c>
       <c r="B364" s="14" t="inlineStr">
@@ -13889,7 +13889,7 @@
     <row r="365">
       <c r="A365" s="14" t="inlineStr">
         <is>
-          <t>Login History as ClearOps_UserLogin</t>
+          <t>Login History as UserLogin</t>
         </is>
       </c>
       <c r="B365" s="15" t="inlineStr">
@@ -13918,7 +13918,7 @@
     <row r="366">
       <c r="A366" s="14" t="inlineStr">
         <is>
-          <t>Login History as ClearOps_UserLogin</t>
+          <t>Login History as UserLogin</t>
         </is>
       </c>
       <c r="B366" s="14" t="inlineStr">
@@ -14307,7 +14307,7 @@
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>Each Pass-through Costs as ClearOps_Passthrough row points to one Project Tasks (WBS) as ClearOps_ProjectWBS row</t>
+          <t>Each Pass-through Costs as ClearOps_Passthrough row points to one Project Tasks (WBS) as ProjectWBS row</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -14322,7 +14322,7 @@
       </c>
       <c r="D15" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="E15" s="13" t="inlineStr">
@@ -14550,12 +14550,12 @@
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>Each Time Off as ClearOps_TimeOff row points to one People (HR master list) as Employee_Master row</t>
+          <t>Each Time Off as TimeOff(WD) row points to one People (HR master list) as Employee_Master row</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>Time Off as ClearOps_TimeOff</t>
+          <t>Time Off as TimeOff(WD)</t>
         </is>
       </c>
       <c r="C24" s="14" t="inlineStr">
@@ -14577,12 +14577,12 @@
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>Each Time Planner as ClearOps_ProjectTimePlanner row points to one Projects as Project_Master row</t>
+          <t>Each Time Planner as ClearOps_Project_Time_Planner row points to one Projects as Project_Master row</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>Time Planner as ClearOps_ProjectTimePlanner</t>
+          <t>Time Planner as ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="C25" s="14" t="inlineStr">
@@ -14604,12 +14604,12 @@
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>Each Time Planner as ClearOps_ProjectTimePlanner row points to one Project Tasks (WBS) as ClearOps_ProjectWBS row</t>
+          <t>Each Time Planner as ClearOps_Project_Time_Planner row points to one Project Tasks (WBS) as ProjectWBS row</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>Time Planner as ClearOps_ProjectTimePlanner</t>
+          <t>Time Planner as ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="C26" s="14" t="inlineStr">
@@ -14619,7 +14619,7 @@
       </c>
       <c r="D26" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="E26" s="16" t="inlineStr">
@@ -14631,12 +14631,12 @@
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>Each Time Planner as ClearOps_ProjectTimePlanner row points to one Resources (bookable people) as Resources row</t>
+          <t>Each Time Planner as ClearOps_Project_Time_Planner row points to one Resources (bookable people) as Resources row</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr">
         <is>
-          <t>Time Planner as ClearOps_ProjectTimePlanner</t>
+          <t>Time Planner as ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="C27" s="14" t="inlineStr">
@@ -14928,12 +14928,12 @@
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>Each Project Tasks (WBS) as ClearOps_ProjectWBS row points to one Projects as Project_Master row</t>
+          <t>Each Project Tasks (WBS) as ProjectWBS row points to one Projects as Project_Master row</t>
         </is>
       </c>
       <c r="B38" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="C38" s="14" t="inlineStr">
@@ -14955,12 +14955,12 @@
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t>Each Project Tasks (WBS) as ClearOps_ProjectWBS row points to one Project Tasks (WBS) as ClearOps_ProjectWBS row</t>
+          <t>Each Project Tasks (WBS) as ProjectWBS row points to one Project Tasks (WBS) as ProjectWBS row</t>
         </is>
       </c>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="C39" s="14" t="inlineStr">
@@ -14970,7 +14970,7 @@
       </c>
       <c r="D39" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="E39" s="13" t="inlineStr">
@@ -14982,12 +14982,12 @@
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t>Each Project Tasks (WBS) as ClearOps_ProjectWBS row points to one Project Tasks (WBS) as ClearOps_ProjectWBS row</t>
+          <t>Each Project Tasks (WBS) as ProjectWBS row points to one Project Tasks (WBS) as ProjectWBS row</t>
         </is>
       </c>
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="C40" s="14" t="inlineStr">
@@ -14997,7 +14997,7 @@
       </c>
       <c r="D40" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="E40" s="16" t="inlineStr">
@@ -15009,12 +15009,12 @@
     <row r="41">
       <c r="A41" s="14" t="inlineStr">
         <is>
-          <t>Each Project Estimates as ClearOps_ProjectEstimator row points to one Projects as Project_Master row</t>
+          <t>Each Project Estimates as Project_Estimator row points to one Projects as Project_Master row</t>
         </is>
       </c>
       <c r="B41" s="14" t="inlineStr">
         <is>
-          <t>Project Estimates as ClearOps_ProjectEstimator</t>
+          <t>Project Estimates as Project_Estimator</t>
         </is>
       </c>
       <c r="C41" s="14" t="inlineStr">
@@ -15036,12 +15036,12 @@
     <row r="42">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>Each Project Estimates as ClearOps_ProjectEstimator row points to one Project Tasks (WBS) as ClearOps_ProjectWBS row</t>
+          <t>Each Project Estimates as Project_Estimator row points to one Project Tasks (WBS) as ProjectWBS row</t>
         </is>
       </c>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>Project Estimates as ClearOps_ProjectEstimator</t>
+          <t>Project Estimates as Project_Estimator</t>
         </is>
       </c>
       <c r="C42" s="14" t="inlineStr">
@@ -15051,7 +15051,7 @@
       </c>
       <c r="D42" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="E42" s="16" t="inlineStr">
@@ -15063,12 +15063,12 @@
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
-          <t>Each Project Estimates as ClearOps_ProjectEstimator row points to one Job Grades as Grades row</t>
+          <t>Each Project Estimates as Project_Estimator row points to one Job Grades as Grades row</t>
         </is>
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>Project Estimates as ClearOps_ProjectEstimator</t>
+          <t>Project Estimates as Project_Estimator</t>
         </is>
       </c>
       <c r="C43" s="14" t="inlineStr">
@@ -15090,12 +15090,12 @@
     <row r="44">
       <c r="A44" s="14" t="inlineStr">
         <is>
-          <t>Each Project Finance Settings as ClearOps_ProjectSettings row points to one Projects as Project_Master row</t>
+          <t>Each Project Finance Settings as Project_Settings row points to one Projects as Project_Master row</t>
         </is>
       </c>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>Project Finance Settings as ClearOps_ProjectSettings</t>
+          <t>Project Finance Settings as Project_Settings</t>
         </is>
       </c>
       <c r="C44" s="14" t="inlineStr">
@@ -15144,7 +15144,7 @@
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
-          <t>Each Project Assignments (grid rows) as ClearOps_ProjectSTP row points to one Project Tasks (WBS) as ClearOps_ProjectWBS row</t>
+          <t>Each Project Assignments (grid rows) as ClearOps_ProjectSTP row points to one Project Tasks (WBS) as ProjectWBS row</t>
         </is>
       </c>
       <c r="B46" s="14" t="inlineStr">
@@ -15159,7 +15159,7 @@
       </c>
       <c r="D46" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="E46" s="16" t="inlineStr">
@@ -15252,12 +15252,12 @@
     <row r="50">
       <c r="A50" s="14" t="inlineStr">
         <is>
-          <t>Each Integration Run Log as ClearOps_Logs row points to one Integration Status as Admin_IntegrationStatus row</t>
+          <t>Each Integration Run Log as Logs_table row points to one Integration Status as Admin_Integration_Status row</t>
         </is>
       </c>
       <c r="B50" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="C50" s="14" t="inlineStr">
@@ -15267,7 +15267,7 @@
       </c>
       <c r="D50" s="14" t="inlineStr">
         <is>
-          <t>Integration Status as Admin_IntegrationStatus</t>
+          <t>Integration Status as Admin_Integration_Status</t>
         </is>
       </c>
       <c r="E50" s="16" t="inlineStr">
@@ -15333,7 +15333,7 @@
     <row r="53">
       <c r="A53" s="14" t="inlineStr">
         <is>
-          <t>Each Permissions as ClearOps_Permission row points to one Access Levels as ClearOps_Access row</t>
+          <t>Each Permissions as ClearOps_Permission row points to one Access Levels as ClearOpps_Access_table row</t>
         </is>
       </c>
       <c r="B53" s="14" t="inlineStr">
@@ -15348,7 +15348,7 @@
       </c>
       <c r="D53" s="14" t="inlineStr">
         <is>
-          <t>Access Levels as ClearOps_Access</t>
+          <t>Access Levels as ClearOpps_Access_table</t>
         </is>
       </c>
       <c r="E53" s="16" t="inlineStr">
@@ -15414,12 +15414,12 @@
     <row r="56">
       <c r="A56" s="14" t="inlineStr">
         <is>
-          <t>Each Single Sign-On Link as ClearOps_Login row points to one People (HR master list) as Employee_Master row</t>
+          <t>Each Single Sign-On Link as ClearOps_login row points to one People (HR master list) as Employee_Master row</t>
         </is>
       </c>
       <c r="B56" s="14" t="inlineStr">
         <is>
-          <t>Single Sign-On Link as ClearOps_Login</t>
+          <t>Single Sign-On Link as ClearOps_login</t>
         </is>
       </c>
       <c r="C56" s="14" t="inlineStr">
@@ -15441,12 +15441,12 @@
     <row r="57">
       <c r="A57" s="14" t="inlineStr">
         <is>
-          <t>Each Login History as ClearOps_UserLogin row points to one Application Users as ClearOps_Users row</t>
+          <t>Each Login History as UserLogin row points to one Application Users as ClearOps_Users row</t>
         </is>
       </c>
       <c r="B57" s="14" t="inlineStr">
         <is>
-          <t>Login History as ClearOps_UserLogin</t>
+          <t>Login History as UserLogin</t>
         </is>
       </c>
       <c r="C57" s="14" t="inlineStr">
@@ -16876,7 +16876,7 @@
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>Time Off as ClearOps_TimeOff</t>
+          <t>Time Off as TimeOff(WD)</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
@@ -16898,7 +16898,7 @@
     <row r="33">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>Time Off as ClearOps_TimeOff</t>
+          <t>Time Off as TimeOff(WD)</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
@@ -16920,7 +16920,7 @@
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>Time Off as ClearOps_TimeOff</t>
+          <t>Time Off as TimeOff(WD)</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
@@ -16942,7 +16942,7 @@
     <row r="35">
       <c r="A35" s="14" t="inlineStr">
         <is>
-          <t>Time Planner as ClearOps_ProjectTimePlanner</t>
+          <t>Time Planner as ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="B35" s="14" t="inlineStr">
@@ -16964,7 +16964,7 @@
     <row r="36">
       <c r="A36" s="14" t="inlineStr">
         <is>
-          <t>Time Planner as ClearOps_ProjectTimePlanner</t>
+          <t>Time Planner as ClearOps_Project_Time_Planner</t>
         </is>
       </c>
       <c r="B36" s="14" t="inlineStr">
@@ -17140,7 +17140,7 @@
     <row r="44">
       <c r="A44" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B44" s="14" t="inlineStr">
@@ -17162,7 +17162,7 @@
     <row r="45">
       <c r="A45" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B45" s="14" t="inlineStr">
@@ -17184,7 +17184,7 @@
     <row r="46">
       <c r="A46" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B46" s="14" t="inlineStr">
@@ -17206,7 +17206,7 @@
     <row r="47">
       <c r="A47" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B47" s="14" t="inlineStr">
@@ -17228,7 +17228,7 @@
     <row r="48">
       <c r="A48" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B48" s="14" t="inlineStr">
@@ -17250,7 +17250,7 @@
     <row r="49">
       <c r="A49" s="14" t="inlineStr">
         <is>
-          <t>Project Tasks (WBS) as ClearOps_ProjectWBS</t>
+          <t>Project Tasks (WBS) as ProjectWBS</t>
         </is>
       </c>
       <c r="B49" s="14" t="inlineStr">
@@ -17272,7 +17272,7 @@
     <row r="50">
       <c r="A50" s="14" t="inlineStr">
         <is>
-          <t>Project Estimates as ClearOps_ProjectEstimator</t>
+          <t>Project Estimates as Project_Estimator</t>
         </is>
       </c>
       <c r="B50" s="14" t="inlineStr">
@@ -17294,7 +17294,7 @@
     <row r="51">
       <c r="A51" s="14" t="inlineStr">
         <is>
-          <t>Project Estimates as ClearOps_ProjectEstimator</t>
+          <t>Project Estimates as Project_Estimator</t>
         </is>
       </c>
       <c r="B51" s="14" t="inlineStr">
@@ -17316,7 +17316,7 @@
     <row r="52">
       <c r="A52" s="14" t="inlineStr">
         <is>
-          <t>Project Estimates as ClearOps_ProjectEstimator</t>
+          <t>Project Estimates as Project_Estimator</t>
         </is>
       </c>
       <c r="B52" s="14" t="inlineStr">
@@ -17338,7 +17338,7 @@
     <row r="53">
       <c r="A53" s="14" t="inlineStr">
         <is>
-          <t>Project Finance Settings as ClearOps_ProjectSettings</t>
+          <t>Project Finance Settings as Project_Settings</t>
         </is>
       </c>
       <c r="B53" s="14" t="inlineStr">
@@ -17360,7 +17360,7 @@
     <row r="54">
       <c r="A54" s="14" t="inlineStr">
         <is>
-          <t>Project Finance Settings as ClearOps_ProjectSettings</t>
+          <t>Project Finance Settings as Project_Settings</t>
         </is>
       </c>
       <c r="B54" s="14" t="inlineStr">
@@ -17558,7 +17558,7 @@
     <row r="63">
       <c r="A63" s="14" t="inlineStr">
         <is>
-          <t>Project Forecasting (OLD) as ClearOps_ProjectForecasting</t>
+          <t>Project Forecasting (OLD) as Project_Forecasting</t>
         </is>
       </c>
       <c r="B63" s="14" t="inlineStr">
@@ -17580,7 +17580,7 @@
     <row r="64">
       <c r="A64" s="14" t="inlineStr">
         <is>
-          <t>Integration Status as Admin_IntegrationStatus</t>
+          <t>Integration Status as Admin_Integration_Status</t>
         </is>
       </c>
       <c r="B64" s="14" t="inlineStr">
@@ -17602,7 +17602,7 @@
     <row r="65">
       <c r="A65" s="14" t="inlineStr">
         <is>
-          <t>Integration Status as Admin_IntegrationStatus</t>
+          <t>Integration Status as Admin_Integration_Status</t>
         </is>
       </c>
       <c r="B65" s="14" t="inlineStr">
@@ -17624,7 +17624,7 @@
     <row r="66">
       <c r="A66" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="B66" s="14" t="inlineStr">
@@ -17646,7 +17646,7 @@
     <row r="67">
       <c r="A67" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="B67" s="14" t="inlineStr">
@@ -17668,7 +17668,7 @@
     <row r="68">
       <c r="A68" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="B68" s="14" t="inlineStr">
@@ -17690,7 +17690,7 @@
     <row r="69">
       <c r="A69" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="B69" s="14" t="inlineStr">
@@ -17712,7 +17712,7 @@
     <row r="70">
       <c r="A70" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="B70" s="14" t="inlineStr">
@@ -17734,7 +17734,7 @@
     <row r="71">
       <c r="A71" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="B71" s="14" t="inlineStr">
@@ -17756,7 +17756,7 @@
     <row r="72">
       <c r="A72" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="B72" s="14" t="inlineStr">
@@ -17778,7 +17778,7 @@
     <row r="73">
       <c r="A73" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="B73" s="14" t="inlineStr">
@@ -17800,7 +17800,7 @@
     <row r="74">
       <c r="A74" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="B74" s="14" t="inlineStr">
@@ -17822,7 +17822,7 @@
     <row r="75">
       <c r="A75" s="14" t="inlineStr">
         <is>
-          <t>Integration Run Log as ClearOps_Logs</t>
+          <t>Integration Run Log as Logs_table</t>
         </is>
       </c>
       <c r="B75" s="14" t="inlineStr">
@@ -17859,7 +17859,7 @@
       </c>
       <c r="D76" s="14" t="inlineStr">
         <is>
-          <t>From RolesandPermissions</t>
+          <t>From ClearOps_RolesandPermissions</t>
         </is>
       </c>
     </row>
@@ -17881,14 +17881,14 @@
       </c>
       <c r="D77" s="14" t="inlineStr">
         <is>
-          <t>Moved from RolesandPermissions</t>
+          <t>Moved from ClearOps_RolesandPermissions</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="14" t="inlineStr">
         <is>
-          <t>Access Levels as ClearOps_Access</t>
+          <t>Access Levels as ClearOpps_Access_table</t>
         </is>
       </c>
       <c r="B78" s="14" t="inlineStr">
@@ -17976,7 +17976,7 @@
     <row r="82">
       <c r="A82" s="14" t="inlineStr">
         <is>
-          <t>Single Sign-On Link as ClearOps_Login</t>
+          <t>Single Sign-On Link as ClearOps_login</t>
         </is>
       </c>
       <c r="B82" s="14" t="inlineStr">
@@ -17998,7 +17998,7 @@
     <row r="83">
       <c r="A83" s="14" t="inlineStr">
         <is>
-          <t>Single Sign-On Link as ClearOps_Login</t>
+          <t>Single Sign-On Link as ClearOps_login</t>
         </is>
       </c>
       <c r="B83" s="14" t="inlineStr">
@@ -18020,7 +18020,7 @@
     <row r="84">
       <c r="A84" s="14" t="inlineStr">
         <is>
-          <t>Single Sign-On Link as ClearOps_Login</t>
+          <t>Single Sign-On Link as ClearOps_login</t>
         </is>
       </c>
       <c r="B84" s="14" t="inlineStr">
@@ -18042,7 +18042,7 @@
     <row r="85">
       <c r="A85" s="14" t="inlineStr">
         <is>
-          <t>Login History as ClearOps_UserLogin</t>
+          <t>Login History as UserLogin</t>
         </is>
       </c>
       <c r="B85" s="14" t="inlineStr">
@@ -18064,7 +18064,7 @@
     <row r="86">
       <c r="A86" s="14" t="inlineStr">
         <is>
-          <t>Login History as ClearOps_UserLogin</t>
+          <t>Login History as UserLogin</t>
         </is>
       </c>
       <c r="B86" s="14" t="inlineStr">
@@ -18086,7 +18086,7 @@
     <row r="87">
       <c r="A87" s="14" t="inlineStr">
         <is>
-          <t>Login History as ClearOps_UserLogin</t>
+          <t>Login History as UserLogin</t>
         </is>
       </c>
       <c r="B87" s="14" t="inlineStr">
@@ -18108,7 +18108,7 @@
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
-          <t>Roles &amp; Permissions (OLD sheet) as RolesandPermissions</t>
+          <t>Roles &amp; Permissions (OLD sheet) as ClearOps_RolesandPermissions</t>
         </is>
       </c>
       <c r="B88" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Rename UserLogin to User_Login in mapping workbook
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A5mSLBPV7GuwkbXJCnEXu9
</commit_message>
<xml_diff>
--- a/ClearOps_Database_Mapped.xlsx
+++ b/ClearOps_Database_Mapped.xlsx
@@ -1458,7 +1458,7 @@
     <row r="48">
       <c r="A48" s="15" t="inlineStr">
         <is>
-          <t>Login History as UserLogin</t>
+          <t>Login History as User_Login</t>
         </is>
       </c>
       <c r="B48" s="14" t="inlineStr">
@@ -2730,7 +2730,7 @@
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>Login History as UserLogin</t>
+          <t>Login History as User_Login</t>
         </is>
       </c>
       <c r="C34" s="15" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>UserLogin</t>
+          <t>User_Login</t>
         </is>
       </c>
       <c r="G34" s="14" t="inlineStr">
@@ -13819,7 +13819,7 @@
     <row r="363">
       <c r="A363" s="14" t="inlineStr">
         <is>
-          <t>Login History as UserLogin</t>
+          <t>Login History as User_Login</t>
         </is>
       </c>
       <c r="B363" s="16" t="inlineStr">
@@ -13839,7 +13839,7 @@
       </c>
       <c r="E363" s="14" t="inlineStr">
         <is>
-          <t>Unique number of each row in Login History as UserLogin [Was missing – no PK]</t>
+          <t>Unique number of each row in Login History as User_Login [Was missing – no PK]</t>
         </is>
       </c>
       <c r="F363" s="14" t="inlineStr">
@@ -13852,7 +13852,7 @@
     <row r="364">
       <c r="A364" s="14" t="inlineStr">
         <is>
-          <t>Login History as UserLogin</t>
+          <t>Login History as User_Login</t>
         </is>
       </c>
       <c r="B364" s="14" t="inlineStr">
@@ -13889,7 +13889,7 @@
     <row r="365">
       <c r="A365" s="14" t="inlineStr">
         <is>
-          <t>Login History as UserLogin</t>
+          <t>Login History as User_Login</t>
         </is>
       </c>
       <c r="B365" s="15" t="inlineStr">
@@ -13918,7 +13918,7 @@
     <row r="366">
       <c r="A366" s="14" t="inlineStr">
         <is>
-          <t>Login History as UserLogin</t>
+          <t>Login History as User_Login</t>
         </is>
       </c>
       <c r="B366" s="14" t="inlineStr">
@@ -15441,12 +15441,12 @@
     <row r="57">
       <c r="A57" s="14" t="inlineStr">
         <is>
-          <t>Each Login History as UserLogin row points to one Application Users as ClearOps_Users row</t>
+          <t>Each Login History as User_Login row points to one Application Users as ClearOps_Users row</t>
         </is>
       </c>
       <c r="B57" s="14" t="inlineStr">
         <is>
-          <t>Login History as UserLogin</t>
+          <t>Login History as User_Login</t>
         </is>
       </c>
       <c r="C57" s="14" t="inlineStr">
@@ -18042,7 +18042,7 @@
     <row r="85">
       <c r="A85" s="14" t="inlineStr">
         <is>
-          <t>Login History as UserLogin</t>
+          <t>Login History as User_Login</t>
         </is>
       </c>
       <c r="B85" s="14" t="inlineStr">
@@ -18064,7 +18064,7 @@
     <row r="86">
       <c r="A86" s="14" t="inlineStr">
         <is>
-          <t>Login History as UserLogin</t>
+          <t>Login History as User_Login</t>
         </is>
       </c>
       <c r="B86" s="14" t="inlineStr">
@@ -18086,7 +18086,7 @@
     <row r="87">
       <c r="A87" s="14" t="inlineStr">
         <is>
-          <t>Login History as UserLogin</t>
+          <t>Login History as User_Login</t>
         </is>
       </c>
       <c r="B87" s="14" t="inlineStr">

</xml_diff>